<commit_message>
Updated DEU model - 2025-09-07 00:07
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_DEU/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3560F2-CE1B-42B9-AA96-E78D0D1B7FF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B17B292A-C922-4554-A347-8D613E547DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="297">
   <si>
     <t>Unit</t>
   </si>
@@ -970,6 +970,9 @@
   </si>
   <si>
     <t>SysCost_Annual</t>
+  </si>
+  <si>
+    <t>f1d</t>
   </si>
 </sst>
 </file>
@@ -4891,11 +4894,11 @@
       </c>
       <c r="C14" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.f3d</v>
+        <v>e 1.5 deg no OS.f1d</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.f3d</v>
+        <v>e 1.5 deg no OS.f1d</v>
       </c>
       <c r="I14" t="str">
         <f t="shared" si="3"/>
@@ -4903,7 +4906,7 @@
       </c>
       <c r="J14" t="str">
         <f t="shared" si="4"/>
-        <v>f3d</v>
+        <v>f1d</v>
       </c>
       <c r="O14">
         <v>9</v>
@@ -5001,7 +5004,7 @@
         <v>263</v>
       </c>
       <c r="U16" t="s">
-        <v>264</v>
+        <v>296</v>
       </c>
     </row>
     <row r="17" spans="2:17">
@@ -5259,11 +5262,11 @@
       </c>
       <c r="C25" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.f3d</v>
+        <v>d 1.5 deg OS.f1d</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.f3d</v>
+        <v>d 1.5 deg OS.f1d</v>
       </c>
       <c r="I25" t="str">
         <f t="shared" si="3"/>
@@ -5271,7 +5274,7 @@
       </c>
       <c r="J25" t="str">
         <f t="shared" si="4"/>
-        <v>f3d</v>
+        <v>f1d</v>
       </c>
       <c r="O25">
         <v>20</v>
@@ -5600,11 +5603,11 @@
       </c>
       <c r="C36" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).f3d</v>
+        <v>c 2 deg (67%).f1d</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).f3d</v>
+        <v>c 2 deg (67%).f1d</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="3"/>
@@ -5612,7 +5615,7 @@
       </c>
       <c r="J36" t="str">
         <f t="shared" si="4"/>
-        <v>f3d</v>
+        <v>f1d</v>
       </c>
       <c r="O36">
         <v>31</v>
@@ -5941,11 +5944,11 @@
       </c>
       <c r="C47" t="str">
         <f t="shared" si="6"/>
-        <v>b 2 deg (50%).f3d</v>
+        <v>b 2 deg (50%).f1d</v>
       </c>
       <c r="H47" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).f3d</v>
+        <v>b 2 deg (50%).f1d</v>
       </c>
       <c r="I47" t="str">
         <f t="shared" si="3"/>
@@ -5953,7 +5956,7 @@
       </c>
       <c r="J47" t="str">
         <f t="shared" si="4"/>
-        <v>f3d</v>
+        <v>f1d</v>
       </c>
       <c r="O47">
         <v>42</v>
@@ -6282,11 +6285,11 @@
       </c>
       <c r="C58" t="str">
         <f t="shared" si="7"/>
-        <v>a 3 deg.f3d</v>
+        <v>a 3 deg.f1d</v>
       </c>
       <c r="H58" t="str">
         <f t="shared" si="8"/>
-        <v>a 3 deg.f3d</v>
+        <v>a 3 deg.f1d</v>
       </c>
       <c r="I58" t="str">
         <f t="shared" si="3"/>
@@ -6294,7 +6297,7 @@
       </c>
       <c r="J58" t="str">
         <f t="shared" si="4"/>
-        <v>f3d</v>
+        <v>f1d</v>
       </c>
       <c r="O58">
         <v>53</v>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-09 22:45
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_DEU/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B17B292A-C922-4554-A347-8D613E547DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC5A96E-17E2-474F-8FC2-5215BD4B5D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -879,9 +879,6 @@
     <t>f3d</t>
   </si>
   <si>
-    <t>~TS_Defs: Snk_attr=SANKEY Grid Flows</t>
-  </si>
-  <si>
     <t>~TS_Defs: Snk_attr=SANKEY whole system</t>
   </si>
   <si>
@@ -973,6 +970,9 @@
   </si>
   <si>
     <t>f1d</t>
+  </si>
+  <si>
+    <t>DeACT TS_Defs: Snk_attr=SANKEY Grid Flows</t>
   </si>
 </sst>
 </file>
@@ -4553,7 +4553,7 @@
         <v>230</v>
       </c>
       <c r="Q6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S6">
         <v>1</v>
@@ -4565,7 +4565,7 @@
         <v>244</v>
       </c>
       <c r="W6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="X6" t="s">
         <v>258</v>
@@ -4602,7 +4602,7 @@
         <v>231</v>
       </c>
       <c r="Q7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S7">
         <v>2</v>
@@ -4614,7 +4614,7 @@
         <v>241</v>
       </c>
       <c r="W7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="X7" t="s">
         <v>257</v>
@@ -4651,7 +4651,7 @@
         <v>232</v>
       </c>
       <c r="Q8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S8">
         <v>3</v>
@@ -4663,7 +4663,7 @@
         <v>242</v>
       </c>
       <c r="W8" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="X8" t="s">
         <v>256</v>
@@ -4700,7 +4700,7 @@
         <v>233</v>
       </c>
       <c r="Q9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S9">
         <v>4</v>
@@ -4712,7 +4712,7 @@
         <v>240</v>
       </c>
       <c r="W9" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="X9" t="s">
         <v>255</v>
@@ -4749,7 +4749,7 @@
         <v>234</v>
       </c>
       <c r="Q10" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S10">
         <v>5</v>
@@ -4761,7 +4761,7 @@
         <v>247</v>
       </c>
       <c r="W10" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="X10" t="s">
         <v>259</v>
@@ -4795,7 +4795,7 @@
         <v>235</v>
       </c>
       <c r="Q11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S11">
         <v>6</v>
@@ -4835,7 +4835,7 @@
         <v>236</v>
       </c>
       <c r="Q12" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S12">
         <v>7</v>
@@ -4875,7 +4875,7 @@
         <v>237</v>
       </c>
       <c r="Q13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S13">
         <v>8</v>
@@ -4915,7 +4915,7 @@
         <v>263</v>
       </c>
       <c r="Q14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S14">
         <v>9</v>
@@ -4955,7 +4955,7 @@
         <v>238</v>
       </c>
       <c r="Q15" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S15">
         <v>10</v>
@@ -4995,7 +4995,7 @@
         <v>239</v>
       </c>
       <c r="Q16" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S16">
         <v>11</v>
@@ -5004,7 +5004,7 @@
         <v>263</v>
       </c>
       <c r="U16" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="17" spans="2:17">
@@ -5035,7 +5035,7 @@
         <v>230</v>
       </c>
       <c r="Q17" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18" spans="2:17">
@@ -5066,7 +5066,7 @@
         <v>231</v>
       </c>
       <c r="Q18" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19" spans="2:17">
@@ -5097,7 +5097,7 @@
         <v>232</v>
       </c>
       <c r="Q19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" spans="2:17">
@@ -5128,7 +5128,7 @@
         <v>233</v>
       </c>
       <c r="Q20" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="21" spans="2:17">
@@ -5159,7 +5159,7 @@
         <v>234</v>
       </c>
       <c r="Q21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="22" spans="2:17">
@@ -5190,7 +5190,7 @@
         <v>235</v>
       </c>
       <c r="Q22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="23" spans="2:17">
@@ -5221,7 +5221,7 @@
         <v>236</v>
       </c>
       <c r="Q23" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="24" spans="2:17">
@@ -5252,7 +5252,7 @@
         <v>237</v>
       </c>
       <c r="Q24" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="25" spans="2:17">
@@ -5283,7 +5283,7 @@
         <v>263</v>
       </c>
       <c r="Q25" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="26" spans="2:17">
@@ -5314,7 +5314,7 @@
         <v>238</v>
       </c>
       <c r="Q26" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="27" spans="2:17">
@@ -5345,7 +5345,7 @@
         <v>239</v>
       </c>
       <c r="Q27" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="28" spans="2:17">
@@ -5376,7 +5376,7 @@
         <v>230</v>
       </c>
       <c r="Q28" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="29" spans="2:17">
@@ -5407,7 +5407,7 @@
         <v>231</v>
       </c>
       <c r="Q29" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="30" spans="2:17">
@@ -5438,7 +5438,7 @@
         <v>232</v>
       </c>
       <c r="Q30" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="31" spans="2:17">
@@ -5469,7 +5469,7 @@
         <v>233</v>
       </c>
       <c r="Q31" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="32" spans="2:17">
@@ -5500,7 +5500,7 @@
         <v>234</v>
       </c>
       <c r="Q32" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="33" spans="2:17">
@@ -5531,7 +5531,7 @@
         <v>235</v>
       </c>
       <c r="Q33" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="34" spans="2:17">
@@ -5562,7 +5562,7 @@
         <v>236</v>
       </c>
       <c r="Q34" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="35" spans="2:17">
@@ -5593,7 +5593,7 @@
         <v>237</v>
       </c>
       <c r="Q35" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="36" spans="2:17">
@@ -5624,7 +5624,7 @@
         <v>263</v>
       </c>
       <c r="Q36" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="37" spans="2:17">
@@ -5655,7 +5655,7 @@
         <v>238</v>
       </c>
       <c r="Q37" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="38" spans="2:17">
@@ -5686,7 +5686,7 @@
         <v>239</v>
       </c>
       <c r="Q38" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="39" spans="2:17">
@@ -5717,7 +5717,7 @@
         <v>230</v>
       </c>
       <c r="Q39" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="40" spans="2:17">
@@ -5748,7 +5748,7 @@
         <v>231</v>
       </c>
       <c r="Q40" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="41" spans="2:17">
@@ -5779,7 +5779,7 @@
         <v>232</v>
       </c>
       <c r="Q41" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="42" spans="2:17">
@@ -5810,7 +5810,7 @@
         <v>233</v>
       </c>
       <c r="Q42" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="43" spans="2:17">
@@ -5841,7 +5841,7 @@
         <v>234</v>
       </c>
       <c r="Q43" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="44" spans="2:17">
@@ -5872,7 +5872,7 @@
         <v>235</v>
       </c>
       <c r="Q44" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="45" spans="2:17">
@@ -5903,7 +5903,7 @@
         <v>236</v>
       </c>
       <c r="Q45" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="46" spans="2:17">
@@ -5934,7 +5934,7 @@
         <v>237</v>
       </c>
       <c r="Q46" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="47" spans="2:17">
@@ -5965,7 +5965,7 @@
         <v>263</v>
       </c>
       <c r="Q47" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="48" spans="2:17">
@@ -5996,7 +5996,7 @@
         <v>238</v>
       </c>
       <c r="Q48" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="49" spans="2:17">
@@ -6027,7 +6027,7 @@
         <v>239</v>
       </c>
       <c r="Q49" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="50" spans="2:17">
@@ -6058,7 +6058,7 @@
         <v>230</v>
       </c>
       <c r="Q50" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="51" spans="2:17">
@@ -6089,7 +6089,7 @@
         <v>231</v>
       </c>
       <c r="Q51" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="52" spans="2:17">
@@ -6120,7 +6120,7 @@
         <v>232</v>
       </c>
       <c r="Q52" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="53" spans="2:17">
@@ -6151,7 +6151,7 @@
         <v>233</v>
       </c>
       <c r="Q53" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="54" spans="2:17">
@@ -6182,7 +6182,7 @@
         <v>234</v>
       </c>
       <c r="Q54" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="55" spans="2:17">
@@ -6213,7 +6213,7 @@
         <v>235</v>
       </c>
       <c r="Q55" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="56" spans="2:17">
@@ -6244,7 +6244,7 @@
         <v>236</v>
       </c>
       <c r="Q56" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="57" spans="2:17">
@@ -6275,7 +6275,7 @@
         <v>237</v>
       </c>
       <c r="Q57" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="58" spans="2:17">
@@ -6306,7 +6306,7 @@
         <v>263</v>
       </c>
       <c r="Q58" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="59" spans="2:17">
@@ -6337,7 +6337,7 @@
         <v>238</v>
       </c>
       <c r="Q59" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="60" spans="2:17">
@@ -6368,7 +6368,7 @@
         <v>239</v>
       </c>
       <c r="Q60" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>
@@ -6605,7 +6605,7 @@
         <v>117</v>
       </c>
       <c r="K9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="N9" t="s">
         <v>82</v>
@@ -6687,13 +6687,13 @@
     </row>
     <row r="14" spans="1:21">
       <c r="A14" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K14" t="s">
+        <v>292</v>
+      </c>
+      <c r="N14" t="s">
         <v>293</v>
-      </c>
-      <c r="N14" t="s">
-        <v>294</v>
       </c>
       <c r="Q14" t="s">
         <v>50</v>
@@ -6701,13 +6701,13 @@
     </row>
     <row r="15" spans="1:21">
       <c r="A15" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="K15" t="s">
         <v>292</v>
       </c>
-      <c r="K15" t="s">
-        <v>293</v>
-      </c>
       <c r="N15" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="Q15" t="s">
         <v>50</v>
@@ -6812,7 +6812,7 @@
   <sheetData>
     <row r="3" spans="1:19" ht="17.25" thickBot="1">
       <c r="A3" s="5" t="s">
-        <v>265</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="15" thickTop="1" thickBot="1">
@@ -6920,7 +6920,7 @@
     </row>
     <row r="10" spans="1:19" ht="17.25" thickBot="1">
       <c r="A10" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="15" thickTop="1" thickBot="1">
@@ -6987,7 +6987,7 @@
         <v>120</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -7006,7 +7006,7 @@
         <v>160</v>
       </c>
       <c r="M13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="S13">
         <v>-1</v>
@@ -7028,7 +7028,7 @@
         <v>160</v>
       </c>
       <c r="M14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="S14">
         <v>-1</v>
@@ -7039,7 +7039,7 @@
         <v>120</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -7058,7 +7058,7 @@
         <v>160</v>
       </c>
       <c r="M16" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="S16">
         <v>-1</v>
@@ -7080,7 +7080,7 @@
         <v>160</v>
       </c>
       <c r="M17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="S17">
         <v>-1</v>
@@ -7091,7 +7091,7 @@
         <v>120</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -7109,7 +7109,7 @@
         <v>160</v>
       </c>
       <c r="M19" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="S19">
         <v>-1</v>
@@ -7130,7 +7130,7 @@
         <v>160</v>
       </c>
       <c r="M20" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="S20">
         <v>-1</v>
@@ -7150,7 +7150,7 @@
         <v>160</v>
       </c>
       <c r="M23" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="S23">
         <v>-1</v>
@@ -7274,7 +7274,7 @@
         <v>94</v>
       </c>
       <c r="B12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -7282,7 +7282,7 @@
         <v>95</v>
       </c>
       <c r="B13" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -7815,7 +7815,7 @@
         <v>202</v>
       </c>
       <c r="B24" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -7823,7 +7823,7 @@
         <v>203</v>
       </c>
       <c r="B25" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -7840,7 +7840,7 @@
         <v>187</v>
       </c>
       <c r="B27" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -7977,7 +7977,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
@@ -7986,7 +7986,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
@@ -8013,7 +8013,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -8022,7 +8022,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -8031,18 +8031,18 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-11 19:15
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_DEU/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC5A96E-17E2-474F-8FC2-5215BD4B5D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBFA3B6F-77C9-4026-A7F7-2B3175ECC1C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="388">
   <si>
     <t>Unit</t>
   </si>
@@ -969,10 +969,283 @@
     <t>SysCost_Annual</t>
   </si>
   <si>
-    <t>f1d</t>
-  </si>
-  <si>
     <t>DeACT TS_Defs: Snk_attr=SANKEY Grid Flows</t>
+  </si>
+  <si>
+    <t>~Scenmap</t>
+  </si>
+  <si>
+    <t>priority</t>
+  </si>
+  <si>
+    <t>scen</t>
+  </si>
+  <si>
+    <t>case_no</t>
+  </si>
+  <si>
+    <t>climate</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.kAnn</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.kAnn</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).kAnn</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).kAnn</t>
+  </si>
+  <si>
+    <t>a 3 deg.kAnn</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.k12</t>
+  </si>
+  <si>
+    <t>ts_12t</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.k12</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).k12</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).k12</t>
+  </si>
+  <si>
+    <t>a 3 deg.k12</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.j12</t>
+  </si>
+  <si>
+    <t>ts_012</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.j12</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).j12</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).j12</t>
+  </si>
+  <si>
+    <t>a 3 deg.j12</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.i24</t>
+  </si>
+  <si>
+    <t>ts_024</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.i24</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).i24</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).i24</t>
+  </si>
+  <si>
+    <t>a 3 deg.i24</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.h48</t>
+  </si>
+  <si>
+    <t>ts_048</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.h48</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).h48</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).h48</t>
+  </si>
+  <si>
+    <t>a 3 deg.h48</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.g64</t>
+  </si>
+  <si>
+    <t>ts_064</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.g64</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).g64</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).g64</t>
+  </si>
+  <si>
+    <t>a 3 deg.g64</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.f97p50</t>
+  </si>
+  <si>
+    <t>ts_096P50</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.f97p50</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).f97p50</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).f97p50</t>
+  </si>
+  <si>
+    <t>a 3 deg.f97p50</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.f96p10</t>
+  </si>
+  <si>
+    <t>ts_096P10</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.f96p10</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).f96p10</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).f96p10</t>
+  </si>
+  <si>
+    <t>a 3 deg.f96p10</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.f96p90</t>
+  </si>
+  <si>
+    <t>ts_096P90</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.f96p90</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).f96p90</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).f96p90</t>
+  </si>
+  <si>
+    <t>a 3 deg.f96p90</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.e3d</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.e3d</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).e3d</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).e3d</t>
+  </si>
+  <si>
+    <t>a 3 deg.e3d</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.d9d</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.d9d</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).d9d</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).d9d</t>
+  </si>
+  <si>
+    <t>a 3 deg.d9d</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.c15d</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.c15d</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).c15d</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).c15d</t>
+  </si>
+  <si>
+    <t>a 3 deg.c15d</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.b2w</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.b2w</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).b2w</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).b2w</t>
+  </si>
+  <si>
+    <t>a 3 deg.b2w</t>
+  </si>
+  <si>
+    <t>e 1.5 deg no OS.a2w2d</t>
+  </si>
+  <si>
+    <t>d 1.5 deg OS.a2w2d</t>
+  </si>
+  <si>
+    <t>c 2 deg (67%).a2w2d</t>
+  </si>
+  <si>
+    <t>b 2 deg (50%).a2w2d</t>
+  </si>
+  <si>
+    <t>a 3 deg.a2w2d</t>
+  </si>
+  <si>
+    <t>kAnn</t>
+  </si>
+  <si>
+    <t>k12</t>
+  </si>
+  <si>
+    <t>j12</t>
+  </si>
+  <si>
+    <t>i24</t>
+  </si>
+  <si>
+    <t>h48</t>
+  </si>
+  <si>
+    <t>g64</t>
+  </si>
+  <si>
+    <t>f97p50</t>
+  </si>
+  <si>
+    <t>f96p10</t>
+  </si>
+  <si>
+    <t>f96p90</t>
   </si>
 </sst>
 </file>
@@ -4455,7 +4728,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet11"/>
-  <dimension ref="B1:X60"/>
+  <dimension ref="B1:X75"/>
   <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="2.73046875" bestFit="1" customWidth="1"/>
@@ -4466,8 +4739,11 @@
     <col min="8" max="8" width="19.59765625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.59765625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.53125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.19921875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.06640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.53125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="2.73046875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="6.33203125" bestFit="1" customWidth="1"/>
@@ -4496,6 +4772,9 @@
       <c r="H4" t="s">
         <v>63</v>
       </c>
+      <c r="O4" t="s">
+        <v>296</v>
+      </c>
     </row>
     <row r="5" spans="2:24">
       <c r="B5" t="s">
@@ -4521,48 +4800,66 @@
         <f>"sg_"&amp;J2</f>
         <v>sg_timeslice</v>
       </c>
+      <c r="N5" t="s">
+        <v>297</v>
+      </c>
+      <c r="O5" t="s">
+        <v>298</v>
+      </c>
+      <c r="P5" t="s">
+        <v>299</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>124</v>
+      </c>
+      <c r="R5" t="s">
+        <v>300</v>
+      </c>
     </row>
     <row r="6" spans="2:24">
       <c r="B6" t="str">
-        <f>"vs~"&amp;TEXT(O6,"0000")</f>
+        <f>"vs~"&amp;TEXT(P6,"0000")</f>
         <v>vs~0001</v>
       </c>
       <c r="C6" t="str">
         <f>H6</f>
-        <v>e 1.5 deg no OS.e3d</v>
+        <v>e 1.5 deg no OS.kAnn</v>
       </c>
       <c r="H6" t="str">
         <f>_xlfn.TEXTJOIN(".",TRUE,I6:J6)</f>
-        <v>e 1.5 deg no OS.e3d</v>
+        <v>e 1.5 deg no OS.kAnn</v>
       </c>
       <c r="I6" t="str">
-        <f>VLOOKUP(Q6,$W$6:$X$12,2,FALSE)</f>
+        <f>VLOOKUP(R6,$W$6:$X$12,2,FALSE)</f>
         <v>e 1.5 deg no OS</v>
       </c>
       <c r="J6" t="str">
-        <f>VLOOKUP(P6,$T$6:$U$16,2,FALSE)</f>
-        <v>e3d</v>
+        <f>VLOOKUP(Q6,$T$6:$U$20,2,FALSE)</f>
+        <v>kAnn</v>
       </c>
       <c r="L6" t="s">
         <v>250</v>
       </c>
-      <c r="O6">
+      <c r="N6">
+        <v>5</v>
+      </c>
+      <c r="O6" t="s">
+        <v>301</v>
+      </c>
+      <c r="P6">
         <v>1</v>
       </c>
-      <c r="P6" t="s">
-        <v>230</v>
-      </c>
       <c r="Q6" t="s">
+        <v>238</v>
+      </c>
+      <c r="R6" t="s">
         <v>285</v>
       </c>
-      <c r="S6">
-        <v>1</v>
-      </c>
       <c r="T6" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="U6" t="s">
-        <v>244</v>
+        <v>379</v>
       </c>
       <c r="W6" t="s">
         <v>285</v>
@@ -4573,45 +4870,48 @@
     </row>
     <row r="7" spans="2:24">
       <c r="B7" t="str">
-        <f t="shared" ref="B7:B60" si="0">"vs~"&amp;TEXT(O7,"0000")</f>
+        <f t="shared" ref="B7:B60" si="0">"vs~"&amp;TEXT(P7,"0000")</f>
         <v>vs~0002</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" ref="C7:C26" si="1">H7</f>
-        <v>e 1.5 deg no OS.d9d</v>
+        <v>d 1.5 deg OS.kAnn</v>
       </c>
       <c r="H7" t="str">
-        <f t="shared" ref="H7:H55" si="2">_xlfn.TEXTJOIN(".",TRUE,I7:J7)</f>
-        <v>e 1.5 deg no OS.d9d</v>
+        <f t="shared" ref="H7:H60" si="2">_xlfn.TEXTJOIN(".",TRUE,I7:J7)</f>
+        <v>d 1.5 deg OS.kAnn</v>
       </c>
       <c r="I7" t="str">
-        <f t="shared" ref="I7:I60" si="3">VLOOKUP(Q7,$W$6:$X$12,2,FALSE)</f>
-        <v>e 1.5 deg no OS</v>
+        <f t="shared" ref="I7:I60" si="3">VLOOKUP(R7,$W$6:$X$12,2,FALSE)</f>
+        <v>d 1.5 deg OS</v>
       </c>
       <c r="J7" t="str">
-        <f t="shared" ref="J7:J60" si="4">VLOOKUP(P7,$T$6:$U$16,2,FALSE)</f>
-        <v>d9d</v>
+        <f t="shared" ref="J7:J60" si="4">VLOOKUP(Q7,$T$6:$U$20,2,FALSE)</f>
+        <v>kAnn</v>
       </c>
       <c r="L7" t="s">
         <v>251</v>
       </c>
-      <c r="O7">
+      <c r="N7">
+        <v>5</v>
+      </c>
+      <c r="O7" t="s">
+        <v>302</v>
+      </c>
+      <c r="P7">
         <v>2</v>
       </c>
-      <c r="P7" t="s">
-        <v>231</v>
-      </c>
       <c r="Q7" t="s">
-        <v>285</v>
-      </c>
-      <c r="S7">
-        <v>2</v>
+        <v>238</v>
+      </c>
+      <c r="R7" t="s">
+        <v>286</v>
       </c>
       <c r="T7" t="s">
-        <v>231</v>
+        <v>307</v>
       </c>
       <c r="U7" t="s">
-        <v>241</v>
+        <v>380</v>
       </c>
       <c r="W7" t="s">
         <v>286</v>
@@ -4627,40 +4927,43 @@
       </c>
       <c r="C8" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.b2w</v>
+        <v>c 2 deg (67%).kAnn</v>
       </c>
       <c r="H8" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.b2w</v>
+        <v>c 2 deg (67%).kAnn</v>
       </c>
       <c r="I8" t="str">
         <f t="shared" si="3"/>
-        <v>e 1.5 deg no OS</v>
+        <v>c 2 deg (67%)</v>
       </c>
       <c r="J8" t="str">
         <f t="shared" si="4"/>
-        <v>b2w</v>
+        <v>kAnn</v>
       </c>
       <c r="L8" t="s">
         <v>252</v>
       </c>
-      <c r="O8">
+      <c r="N8">
+        <v>5</v>
+      </c>
+      <c r="O8" t="s">
+        <v>303</v>
+      </c>
+      <c r="P8">
         <v>3</v>
       </c>
-      <c r="P8" t="s">
-        <v>232</v>
-      </c>
       <c r="Q8" t="s">
-        <v>285</v>
-      </c>
-      <c r="S8">
-        <v>3</v>
+        <v>238</v>
+      </c>
+      <c r="R8" t="s">
+        <v>287</v>
       </c>
       <c r="T8" t="s">
-        <v>232</v>
+        <v>313</v>
       </c>
       <c r="U8" t="s">
-        <v>242</v>
+        <v>381</v>
       </c>
       <c r="W8" t="s">
         <v>287</v>
@@ -4676,40 +4979,43 @@
       </c>
       <c r="C9" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.a2w2d</v>
+        <v>b 2 deg (50%).kAnn</v>
       </c>
       <c r="H9" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.a2w2d</v>
+        <v>b 2 deg (50%).kAnn</v>
       </c>
       <c r="I9" t="str">
         <f t="shared" si="3"/>
-        <v>e 1.5 deg no OS</v>
+        <v>b 2 deg (50%)</v>
       </c>
       <c r="J9" t="str">
         <f t="shared" si="4"/>
-        <v>a2w2d</v>
+        <v>kAnn</v>
       </c>
       <c r="L9" t="s">
         <v>253</v>
       </c>
-      <c r="O9">
+      <c r="N9">
+        <v>5</v>
+      </c>
+      <c r="O9" t="s">
+        <v>304</v>
+      </c>
+      <c r="P9">
         <v>4</v>
       </c>
-      <c r="P9" t="s">
-        <v>233</v>
-      </c>
       <c r="Q9" t="s">
-        <v>285</v>
-      </c>
-      <c r="S9">
-        <v>4</v>
+        <v>238</v>
+      </c>
+      <c r="R9" t="s">
+        <v>288</v>
       </c>
       <c r="T9" t="s">
-        <v>233</v>
+        <v>319</v>
       </c>
       <c r="U9" t="s">
-        <v>240</v>
+        <v>382</v>
       </c>
       <c r="W9" t="s">
         <v>288</v>
@@ -4725,40 +5031,43 @@
       </c>
       <c r="C10" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.hTS12c</v>
+        <v>a 3 deg.kAnn</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.hTS12c</v>
+        <v>a 3 deg.kAnn</v>
       </c>
       <c r="I10" t="str">
         <f t="shared" si="3"/>
-        <v>e 1.5 deg no OS</v>
+        <v>a 3 deg</v>
       </c>
       <c r="J10" t="str">
         <f t="shared" si="4"/>
-        <v>hTS12c</v>
+        <v>kAnn</v>
       </c>
       <c r="L10" t="s">
         <v>254</v>
       </c>
-      <c r="O10">
-        <v>5</v>
-      </c>
-      <c r="P10" t="s">
-        <v>234</v>
+      <c r="N10">
+        <v>5</v>
+      </c>
+      <c r="O10" t="s">
+        <v>305</v>
+      </c>
+      <c r="P10">
+        <v>5</v>
       </c>
       <c r="Q10" t="s">
-        <v>285</v>
-      </c>
-      <c r="S10">
-        <v>5</v>
+        <v>238</v>
+      </c>
+      <c r="R10" t="s">
+        <v>289</v>
       </c>
       <c r="T10" t="s">
-        <v>234</v>
+        <v>325</v>
       </c>
       <c r="U10" t="s">
-        <v>247</v>
+        <v>383</v>
       </c>
       <c r="W10" t="s">
         <v>289</v>
@@ -4774,11 +5083,11 @@
       </c>
       <c r="C11" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.gTS24c</v>
+        <v>e 1.5 deg no OS.k12</v>
       </c>
       <c r="H11" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.gTS24c</v>
+        <v>e 1.5 deg no OS.k12</v>
       </c>
       <c r="I11" t="str">
         <f t="shared" si="3"/>
@@ -4786,25 +5095,28 @@
       </c>
       <c r="J11" t="str">
         <f t="shared" si="4"/>
-        <v>gTS24c</v>
-      </c>
-      <c r="O11">
+        <v>k12</v>
+      </c>
+      <c r="N11">
+        <v>5</v>
+      </c>
+      <c r="O11" t="s">
+        <v>306</v>
+      </c>
+      <c r="P11">
         <v>6</v>
       </c>
-      <c r="P11" t="s">
-        <v>235</v>
-      </c>
       <c r="Q11" t="s">
+        <v>307</v>
+      </c>
+      <c r="R11" t="s">
         <v>285</v>
       </c>
-      <c r="S11">
-        <v>6</v>
-      </c>
       <c r="T11" t="s">
-        <v>235</v>
+        <v>331</v>
       </c>
       <c r="U11" t="s">
-        <v>246</v>
+        <v>384</v>
       </c>
     </row>
     <row r="12" spans="2:24">
@@ -4814,37 +5126,40 @@
       </c>
       <c r="C12" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.fTS48c</v>
+        <v>d 1.5 deg OS.k12</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.fTS48c</v>
+        <v>d 1.5 deg OS.k12</v>
       </c>
       <c r="I12" t="str">
         <f t="shared" si="3"/>
-        <v>e 1.5 deg no OS</v>
+        <v>d 1.5 deg OS</v>
       </c>
       <c r="J12" t="str">
         <f t="shared" si="4"/>
-        <v>fTS48c</v>
-      </c>
-      <c r="O12">
+        <v>k12</v>
+      </c>
+      <c r="N12">
+        <v>5</v>
+      </c>
+      <c r="O12" t="s">
+        <v>308</v>
+      </c>
+      <c r="P12">
         <v>7</v>
       </c>
-      <c r="P12" t="s">
-        <v>236</v>
-      </c>
       <c r="Q12" t="s">
-        <v>285</v>
-      </c>
-      <c r="S12">
-        <v>7</v>
+        <v>307</v>
+      </c>
+      <c r="R12" t="s">
+        <v>286</v>
       </c>
       <c r="T12" t="s">
-        <v>236</v>
+        <v>337</v>
       </c>
       <c r="U12" t="s">
-        <v>245</v>
+        <v>385</v>
       </c>
     </row>
     <row r="13" spans="2:24">
@@ -4854,37 +5169,40 @@
       </c>
       <c r="C13" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.c15d</v>
+        <v>c 2 deg (67%).k12</v>
       </c>
       <c r="H13" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.c15d</v>
+        <v>c 2 deg (67%).k12</v>
       </c>
       <c r="I13" t="str">
         <f t="shared" si="3"/>
-        <v>e 1.5 deg no OS</v>
+        <v>c 2 deg (67%)</v>
       </c>
       <c r="J13" t="str">
         <f t="shared" si="4"/>
-        <v>c15d</v>
-      </c>
-      <c r="O13">
+        <v>k12</v>
+      </c>
+      <c r="N13">
+        <v>5</v>
+      </c>
+      <c r="O13" t="s">
+        <v>309</v>
+      </c>
+      <c r="P13">
         <v>8</v>
       </c>
-      <c r="P13" t="s">
-        <v>237</v>
-      </c>
       <c r="Q13" t="s">
-        <v>285</v>
-      </c>
-      <c r="S13">
-        <v>8</v>
+        <v>307</v>
+      </c>
+      <c r="R13" t="s">
+        <v>287</v>
       </c>
       <c r="T13" t="s">
-        <v>237</v>
+        <v>343</v>
       </c>
       <c r="U13" t="s">
-        <v>243</v>
+        <v>386</v>
       </c>
     </row>
     <row r="14" spans="2:24">
@@ -4894,37 +5212,40 @@
       </c>
       <c r="C14" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.f1d</v>
+        <v>b 2 deg (50%).k12</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.f1d</v>
+        <v>b 2 deg (50%).k12</v>
       </c>
       <c r="I14" t="str">
         <f t="shared" si="3"/>
-        <v>e 1.5 deg no OS</v>
+        <v>b 2 deg (50%)</v>
       </c>
       <c r="J14" t="str">
         <f t="shared" si="4"/>
-        <v>f1d</v>
-      </c>
-      <c r="O14">
+        <v>k12</v>
+      </c>
+      <c r="N14">
+        <v>5</v>
+      </c>
+      <c r="O14" t="s">
+        <v>310</v>
+      </c>
+      <c r="P14">
         <v>9</v>
       </c>
-      <c r="P14" t="s">
-        <v>263</v>
-      </c>
       <c r="Q14" t="s">
-        <v>285</v>
-      </c>
-      <c r="S14">
-        <v>9</v>
+        <v>307</v>
+      </c>
+      <c r="R14" t="s">
+        <v>288</v>
       </c>
       <c r="T14" t="s">
-        <v>239</v>
+        <v>349</v>
       </c>
       <c r="U14" t="s">
-        <v>248</v>
+        <v>387</v>
       </c>
     </row>
     <row r="15" spans="2:24">
@@ -4934,37 +5255,40 @@
       </c>
       <c r="C15" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.jAnn</v>
+        <v>a 3 deg.k12</v>
       </c>
       <c r="H15" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.jAnn</v>
+        <v>a 3 deg.k12</v>
       </c>
       <c r="I15" t="str">
         <f t="shared" si="3"/>
-        <v>e 1.5 deg no OS</v>
+        <v>a 3 deg</v>
       </c>
       <c r="J15" t="str">
         <f t="shared" si="4"/>
-        <v>jAnn</v>
-      </c>
-      <c r="O15">
+        <v>k12</v>
+      </c>
+      <c r="N15">
+        <v>5</v>
+      </c>
+      <c r="O15" t="s">
+        <v>311</v>
+      </c>
+      <c r="P15">
         <v>10</v>
       </c>
-      <c r="P15" t="s">
-        <v>238</v>
-      </c>
       <c r="Q15" t="s">
-        <v>285</v>
-      </c>
-      <c r="S15">
-        <v>10</v>
+        <v>307</v>
+      </c>
+      <c r="R15" t="s">
+        <v>289</v>
       </c>
       <c r="T15" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="U15" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="16" spans="2:24">
@@ -4974,11 +5298,11 @@
       </c>
       <c r="C16" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.iTS12</v>
+        <v>e 1.5 deg no OS.j12</v>
       </c>
       <c r="H16" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.iTS12</v>
+        <v>e 1.5 deg no OS.j12</v>
       </c>
       <c r="I16" t="str">
         <f t="shared" si="3"/>
@@ -4986,39 +5310,42 @@
       </c>
       <c r="J16" t="str">
         <f t="shared" si="4"/>
-        <v>iTS12</v>
-      </c>
-      <c r="O16">
+        <v>j12</v>
+      </c>
+      <c r="N16">
+        <v>5</v>
+      </c>
+      <c r="O16" t="s">
+        <v>312</v>
+      </c>
+      <c r="P16">
         <v>11</v>
       </c>
-      <c r="P16" t="s">
-        <v>239</v>
-      </c>
       <c r="Q16" t="s">
+        <v>313</v>
+      </c>
+      <c r="R16" t="s">
         <v>285</v>
       </c>
-      <c r="S16">
-        <v>11</v>
-      </c>
       <c r="T16" t="s">
-        <v>263</v>
+        <v>231</v>
       </c>
       <c r="U16" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="17" spans="2:17">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="17" spans="2:21">
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>vs~0012</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.e3d</v>
+        <v>d 1.5 deg OS.j12</v>
       </c>
       <c r="H17" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.e3d</v>
+        <v>d 1.5 deg OS.j12</v>
       </c>
       <c r="I17" t="str">
         <f t="shared" si="3"/>
@@ -5026,154 +5353,202 @@
       </c>
       <c r="J17" t="str">
         <f t="shared" si="4"/>
-        <v>e3d</v>
-      </c>
-      <c r="O17">
+        <v>j12</v>
+      </c>
+      <c r="N17">
+        <v>5</v>
+      </c>
+      <c r="O17" t="s">
+        <v>314</v>
+      </c>
+      <c r="P17">
         <v>12</v>
       </c>
-      <c r="P17" t="s">
-        <v>230</v>
-      </c>
       <c r="Q17" t="s">
+        <v>313</v>
+      </c>
+      <c r="R17" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="18" spans="2:17">
+      <c r="T17" t="s">
+        <v>237</v>
+      </c>
+      <c r="U17" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="18" spans="2:21">
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>vs~0013</v>
       </c>
       <c r="C18" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.d9d</v>
+        <v>c 2 deg (67%).j12</v>
       </c>
       <c r="H18" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.d9d</v>
+        <v>c 2 deg (67%).j12</v>
       </c>
       <c r="I18" t="str">
         <f t="shared" si="3"/>
-        <v>d 1.5 deg OS</v>
+        <v>c 2 deg (67%)</v>
       </c>
       <c r="J18" t="str">
         <f t="shared" si="4"/>
-        <v>d9d</v>
-      </c>
-      <c r="O18">
+        <v>j12</v>
+      </c>
+      <c r="N18">
+        <v>5</v>
+      </c>
+      <c r="O18" t="s">
+        <v>315</v>
+      </c>
+      <c r="P18">
         <v>13</v>
       </c>
-      <c r="P18" t="s">
-        <v>231</v>
-      </c>
       <c r="Q18" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="19" spans="2:17">
+        <v>313</v>
+      </c>
+      <c r="R18" t="s">
+        <v>287</v>
+      </c>
+      <c r="T18" t="s">
+        <v>232</v>
+      </c>
+      <c r="U18" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="19" spans="2:21">
       <c r="B19" t="str">
         <f t="shared" si="0"/>
         <v>vs~0014</v>
       </c>
       <c r="C19" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.b2w</v>
+        <v>b 2 deg (50%).j12</v>
       </c>
       <c r="H19" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.b2w</v>
+        <v>b 2 deg (50%).j12</v>
       </c>
       <c r="I19" t="str">
         <f t="shared" si="3"/>
-        <v>d 1.5 deg OS</v>
+        <v>b 2 deg (50%)</v>
       </c>
       <c r="J19" t="str">
         <f t="shared" si="4"/>
-        <v>b2w</v>
-      </c>
-      <c r="O19">
+        <v>j12</v>
+      </c>
+      <c r="N19">
+        <v>5</v>
+      </c>
+      <c r="O19" t="s">
+        <v>316</v>
+      </c>
+      <c r="P19">
         <v>14</v>
       </c>
-      <c r="P19" t="s">
-        <v>232</v>
-      </c>
       <c r="Q19" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="20" spans="2:17">
+        <v>313</v>
+      </c>
+      <c r="R19" t="s">
+        <v>288</v>
+      </c>
+      <c r="T19" t="s">
+        <v>233</v>
+      </c>
+      <c r="U19" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="20" spans="2:21">
       <c r="B20" t="str">
         <f t="shared" si="0"/>
         <v>vs~0015</v>
       </c>
       <c r="C20" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.a2w2d</v>
+        <v>a 3 deg.j12</v>
       </c>
       <c r="H20" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.a2w2d</v>
+        <v>a 3 deg.j12</v>
       </c>
       <c r="I20" t="str">
         <f t="shared" si="3"/>
-        <v>d 1.5 deg OS</v>
+        <v>a 3 deg</v>
       </c>
       <c r="J20" t="str">
         <f t="shared" si="4"/>
-        <v>a2w2d</v>
-      </c>
-      <c r="O20">
+        <v>j12</v>
+      </c>
+      <c r="N20">
+        <v>5</v>
+      </c>
+      <c r="O20" t="s">
+        <v>317</v>
+      </c>
+      <c r="P20">
         <v>15</v>
       </c>
-      <c r="P20" t="s">
-        <v>233</v>
-      </c>
       <c r="Q20" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="21" spans="2:17">
+        <v>313</v>
+      </c>
+      <c r="R20" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="21" spans="2:21">
       <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v>vs~0016</v>
       </c>
       <c r="C21" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.hTS12c</v>
+        <v>e 1.5 deg no OS.i24</v>
       </c>
       <c r="H21" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.hTS12c</v>
+        <v>e 1.5 deg no OS.i24</v>
       </c>
       <c r="I21" t="str">
         <f t="shared" si="3"/>
-        <v>d 1.5 deg OS</v>
+        <v>e 1.5 deg no OS</v>
       </c>
       <c r="J21" t="str">
         <f t="shared" si="4"/>
-        <v>hTS12c</v>
-      </c>
-      <c r="O21">
+        <v>i24</v>
+      </c>
+      <c r="N21">
+        <v>5</v>
+      </c>
+      <c r="O21" t="s">
+        <v>318</v>
+      </c>
+      <c r="P21">
         <v>16</v>
       </c>
-      <c r="P21" t="s">
-        <v>234</v>
-      </c>
       <c r="Q21" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="22" spans="2:17">
+        <v>319</v>
+      </c>
+      <c r="R21" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="22" spans="2:21">
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>vs~0017</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.gTS24c</v>
+        <v>d 1.5 deg OS.i24</v>
       </c>
       <c r="H22" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.gTS24c</v>
+        <v>d 1.5 deg OS.i24</v>
       </c>
       <c r="I22" t="str">
         <f t="shared" si="3"/>
@@ -5181,154 +5556,184 @@
       </c>
       <c r="J22" t="str">
         <f t="shared" si="4"/>
-        <v>gTS24c</v>
-      </c>
-      <c r="O22">
+        <v>i24</v>
+      </c>
+      <c r="N22">
+        <v>5</v>
+      </c>
+      <c r="O22" t="s">
+        <v>320</v>
+      </c>
+      <c r="P22">
         <v>17</v>
       </c>
-      <c r="P22" t="s">
-        <v>235</v>
-      </c>
       <c r="Q22" t="s">
+        <v>319</v>
+      </c>
+      <c r="R22" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="23" spans="2:17">
+    <row r="23" spans="2:21">
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>vs~0018</v>
       </c>
       <c r="C23" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.fTS48c</v>
+        <v>c 2 deg (67%).i24</v>
       </c>
       <c r="H23" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.fTS48c</v>
+        <v>c 2 deg (67%).i24</v>
       </c>
       <c r="I23" t="str">
         <f t="shared" si="3"/>
-        <v>d 1.5 deg OS</v>
+        <v>c 2 deg (67%)</v>
       </c>
       <c r="J23" t="str">
         <f t="shared" si="4"/>
-        <v>fTS48c</v>
-      </c>
-      <c r="O23">
+        <v>i24</v>
+      </c>
+      <c r="N23">
+        <v>5</v>
+      </c>
+      <c r="O23" t="s">
+        <v>321</v>
+      </c>
+      <c r="P23">
         <v>18</v>
       </c>
-      <c r="P23" t="s">
-        <v>236</v>
-      </c>
       <c r="Q23" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="24" spans="2:17">
+        <v>319</v>
+      </c>
+      <c r="R23" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="24" spans="2:21">
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>vs~0019</v>
       </c>
       <c r="C24" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.c15d</v>
+        <v>b 2 deg (50%).i24</v>
       </c>
       <c r="H24" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.c15d</v>
+        <v>b 2 deg (50%).i24</v>
       </c>
       <c r="I24" t="str">
         <f t="shared" si="3"/>
-        <v>d 1.5 deg OS</v>
+        <v>b 2 deg (50%)</v>
       </c>
       <c r="J24" t="str">
         <f t="shared" si="4"/>
-        <v>c15d</v>
-      </c>
-      <c r="O24">
+        <v>i24</v>
+      </c>
+      <c r="N24">
+        <v>5</v>
+      </c>
+      <c r="O24" t="s">
+        <v>322</v>
+      </c>
+      <c r="P24">
         <v>19</v>
       </c>
-      <c r="P24" t="s">
-        <v>237</v>
-      </c>
       <c r="Q24" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="25" spans="2:17">
+        <v>319</v>
+      </c>
+      <c r="R24" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="25" spans="2:21">
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>vs~0020</v>
       </c>
       <c r="C25" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.f1d</v>
+        <v>a 3 deg.i24</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.f1d</v>
+        <v>a 3 deg.i24</v>
       </c>
       <c r="I25" t="str">
         <f t="shared" si="3"/>
-        <v>d 1.5 deg OS</v>
+        <v>a 3 deg</v>
       </c>
       <c r="J25" t="str">
         <f t="shared" si="4"/>
-        <v>f1d</v>
-      </c>
-      <c r="O25">
+        <v>i24</v>
+      </c>
+      <c r="N25">
+        <v>5</v>
+      </c>
+      <c r="O25" t="s">
+        <v>323</v>
+      </c>
+      <c r="P25">
         <v>20</v>
       </c>
-      <c r="P25" t="s">
-        <v>263</v>
-      </c>
       <c r="Q25" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="26" spans="2:17">
+        <v>319</v>
+      </c>
+      <c r="R25" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="26" spans="2:21">
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v>vs~0021</v>
       </c>
       <c r="C26" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.jAnn</v>
+        <v>e 1.5 deg no OS.h48</v>
       </c>
       <c r="H26" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.jAnn</v>
+        <v>e 1.5 deg no OS.h48</v>
       </c>
       <c r="I26" t="str">
         <f t="shared" si="3"/>
-        <v>d 1.5 deg OS</v>
+        <v>e 1.5 deg no OS</v>
       </c>
       <c r="J26" t="str">
         <f t="shared" si="4"/>
-        <v>jAnn</v>
-      </c>
-      <c r="O26">
+        <v>h48</v>
+      </c>
+      <c r="N26">
+        <v>5</v>
+      </c>
+      <c r="O26" t="s">
+        <v>324</v>
+      </c>
+      <c r="P26">
         <v>21</v>
       </c>
-      <c r="P26" t="s">
-        <v>238</v>
-      </c>
       <c r="Q26" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="27" spans="2:17">
+        <v>325</v>
+      </c>
+      <c r="R26" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="27" spans="2:21">
       <c r="B27" t="str">
         <f t="shared" si="0"/>
         <v>vs~0022</v>
       </c>
       <c r="C27" t="str">
         <f t="shared" ref="C27:C40" si="5">H27</f>
-        <v>d 1.5 deg OS.iTS12</v>
+        <v>d 1.5 deg OS.h48</v>
       </c>
       <c r="H27" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.iTS12</v>
+        <v>d 1.5 deg OS.h48</v>
       </c>
       <c r="I27" t="str">
         <f t="shared" si="3"/>
@@ -5336,30 +5741,36 @@
       </c>
       <c r="J27" t="str">
         <f t="shared" si="4"/>
-        <v>iTS12</v>
-      </c>
-      <c r="O27">
+        <v>h48</v>
+      </c>
+      <c r="N27">
+        <v>5</v>
+      </c>
+      <c r="O27" t="s">
+        <v>326</v>
+      </c>
+      <c r="P27">
         <v>22</v>
       </c>
-      <c r="P27" t="s">
-        <v>239</v>
-      </c>
       <c r="Q27" t="s">
+        <v>325</v>
+      </c>
+      <c r="R27" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="28" spans="2:17">
+    <row r="28" spans="2:21">
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>vs~0023</v>
       </c>
       <c r="C28" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).e3d</v>
+        <v>c 2 deg (67%).h48</v>
       </c>
       <c r="H28" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).e3d</v>
+        <v>c 2 deg (67%).h48</v>
       </c>
       <c r="I28" t="str">
         <f t="shared" si="3"/>
@@ -5367,154 +5778,184 @@
       </c>
       <c r="J28" t="str">
         <f t="shared" si="4"/>
-        <v>e3d</v>
-      </c>
-      <c r="O28">
+        <v>h48</v>
+      </c>
+      <c r="N28">
+        <v>5</v>
+      </c>
+      <c r="O28" t="s">
+        <v>327</v>
+      </c>
+      <c r="P28">
         <v>23</v>
       </c>
-      <c r="P28" t="s">
-        <v>230</v>
-      </c>
       <c r="Q28" t="s">
+        <v>325</v>
+      </c>
+      <c r="R28" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="29" spans="2:17">
+    <row r="29" spans="2:21">
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>vs~0024</v>
       </c>
       <c r="C29" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).d9d</v>
+        <v>b 2 deg (50%).h48</v>
       </c>
       <c r="H29" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).d9d</v>
+        <v>b 2 deg (50%).h48</v>
       </c>
       <c r="I29" t="str">
         <f t="shared" si="3"/>
-        <v>c 2 deg (67%)</v>
+        <v>b 2 deg (50%)</v>
       </c>
       <c r="J29" t="str">
         <f t="shared" si="4"/>
-        <v>d9d</v>
-      </c>
-      <c r="O29">
+        <v>h48</v>
+      </c>
+      <c r="N29">
+        <v>5</v>
+      </c>
+      <c r="O29" t="s">
+        <v>328</v>
+      </c>
+      <c r="P29">
         <v>24</v>
       </c>
-      <c r="P29" t="s">
-        <v>231</v>
-      </c>
       <c r="Q29" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="30" spans="2:17">
+        <v>325</v>
+      </c>
+      <c r="R29" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="30" spans="2:21">
       <c r="B30" t="str">
         <f t="shared" si="0"/>
         <v>vs~0025</v>
       </c>
       <c r="C30" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).b2w</v>
+        <v>a 3 deg.h48</v>
       </c>
       <c r="H30" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).b2w</v>
+        <v>a 3 deg.h48</v>
       </c>
       <c r="I30" t="str">
         <f t="shared" si="3"/>
-        <v>c 2 deg (67%)</v>
+        <v>a 3 deg</v>
       </c>
       <c r="J30" t="str">
         <f t="shared" si="4"/>
-        <v>b2w</v>
-      </c>
-      <c r="O30">
+        <v>h48</v>
+      </c>
+      <c r="N30">
+        <v>5</v>
+      </c>
+      <c r="O30" t="s">
+        <v>329</v>
+      </c>
+      <c r="P30">
         <v>25</v>
       </c>
-      <c r="P30" t="s">
-        <v>232</v>
-      </c>
       <c r="Q30" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="31" spans="2:17">
+        <v>325</v>
+      </c>
+      <c r="R30" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="31" spans="2:21">
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>vs~0026</v>
       </c>
       <c r="C31" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).a2w2d</v>
+        <v>e 1.5 deg no OS.g64</v>
       </c>
       <c r="H31" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).a2w2d</v>
+        <v>e 1.5 deg no OS.g64</v>
       </c>
       <c r="I31" t="str">
         <f t="shared" si="3"/>
-        <v>c 2 deg (67%)</v>
+        <v>e 1.5 deg no OS</v>
       </c>
       <c r="J31" t="str">
         <f t="shared" si="4"/>
-        <v>a2w2d</v>
-      </c>
-      <c r="O31">
+        <v>g64</v>
+      </c>
+      <c r="N31">
+        <v>5</v>
+      </c>
+      <c r="O31" t="s">
+        <v>330</v>
+      </c>
+      <c r="P31">
         <v>26</v>
       </c>
-      <c r="P31" t="s">
-        <v>233</v>
-      </c>
       <c r="Q31" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="32" spans="2:17">
+        <v>331</v>
+      </c>
+      <c r="R31" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="32" spans="2:21">
       <c r="B32" t="str">
         <f t="shared" si="0"/>
         <v>vs~0027</v>
       </c>
       <c r="C32" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).hTS12c</v>
+        <v>d 1.5 deg OS.g64</v>
       </c>
       <c r="H32" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).hTS12c</v>
+        <v>d 1.5 deg OS.g64</v>
       </c>
       <c r="I32" t="str">
         <f t="shared" si="3"/>
-        <v>c 2 deg (67%)</v>
+        <v>d 1.5 deg OS</v>
       </c>
       <c r="J32" t="str">
         <f t="shared" si="4"/>
-        <v>hTS12c</v>
-      </c>
-      <c r="O32">
+        <v>g64</v>
+      </c>
+      <c r="N32">
+        <v>5</v>
+      </c>
+      <c r="O32" t="s">
+        <v>332</v>
+      </c>
+      <c r="P32">
         <v>27</v>
       </c>
-      <c r="P32" t="s">
-        <v>234</v>
-      </c>
       <c r="Q32" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="33" spans="2:17">
+        <v>331</v>
+      </c>
+      <c r="R32" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="33" spans="2:18">
       <c r="B33" t="str">
         <f t="shared" si="0"/>
         <v>vs~0028</v>
       </c>
       <c r="C33" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).gTS24c</v>
+        <v>c 2 deg (67%).g64</v>
       </c>
       <c r="H33" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).gTS24c</v>
+        <v>c 2 deg (67%).g64</v>
       </c>
       <c r="I33" t="str">
         <f t="shared" si="3"/>
@@ -5522,154 +5963,184 @@
       </c>
       <c r="J33" t="str">
         <f t="shared" si="4"/>
-        <v>gTS24c</v>
-      </c>
-      <c r="O33">
+        <v>g64</v>
+      </c>
+      <c r="N33">
+        <v>5</v>
+      </c>
+      <c r="O33" t="s">
+        <v>333</v>
+      </c>
+      <c r="P33">
         <v>28</v>
       </c>
-      <c r="P33" t="s">
-        <v>235</v>
-      </c>
       <c r="Q33" t="s">
+        <v>331</v>
+      </c>
+      <c r="R33" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="34" spans="2:17">
+    <row r="34" spans="2:18">
       <c r="B34" t="str">
         <f t="shared" si="0"/>
         <v>vs~0029</v>
       </c>
       <c r="C34" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).fTS48c</v>
+        <v>b 2 deg (50%).g64</v>
       </c>
       <c r="H34" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).fTS48c</v>
+        <v>b 2 deg (50%).g64</v>
       </c>
       <c r="I34" t="str">
         <f t="shared" si="3"/>
-        <v>c 2 deg (67%)</v>
+        <v>b 2 deg (50%)</v>
       </c>
       <c r="J34" t="str">
         <f t="shared" si="4"/>
-        <v>fTS48c</v>
-      </c>
-      <c r="O34">
+        <v>g64</v>
+      </c>
+      <c r="N34">
+        <v>5</v>
+      </c>
+      <c r="O34" t="s">
+        <v>334</v>
+      </c>
+      <c r="P34">
         <v>29</v>
       </c>
-      <c r="P34" t="s">
-        <v>236</v>
-      </c>
       <c r="Q34" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="35" spans="2:17">
+        <v>331</v>
+      </c>
+      <c r="R34" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="35" spans="2:18">
       <c r="B35" t="str">
         <f t="shared" si="0"/>
         <v>vs~0030</v>
       </c>
       <c r="C35" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).c15d</v>
+        <v>a 3 deg.g64</v>
       </c>
       <c r="H35" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).c15d</v>
+        <v>a 3 deg.g64</v>
       </c>
       <c r="I35" t="str">
         <f t="shared" si="3"/>
-        <v>c 2 deg (67%)</v>
+        <v>a 3 deg</v>
       </c>
       <c r="J35" t="str">
         <f t="shared" si="4"/>
-        <v>c15d</v>
-      </c>
-      <c r="O35">
+        <v>g64</v>
+      </c>
+      <c r="N35">
+        <v>5</v>
+      </c>
+      <c r="O35" t="s">
+        <v>335</v>
+      </c>
+      <c r="P35">
         <v>30</v>
       </c>
-      <c r="P35" t="s">
-        <v>237</v>
-      </c>
       <c r="Q35" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="36" spans="2:17">
+        <v>331</v>
+      </c>
+      <c r="R35" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="36" spans="2:18">
       <c r="B36" t="str">
         <f t="shared" si="0"/>
         <v>vs~0031</v>
       </c>
       <c r="C36" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).f1d</v>
+        <v>e 1.5 deg no OS.f97p50</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).f1d</v>
+        <v>e 1.5 deg no OS.f97p50</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="3"/>
-        <v>c 2 deg (67%)</v>
+        <v>e 1.5 deg no OS</v>
       </c>
       <c r="J36" t="str">
         <f t="shared" si="4"/>
-        <v>f1d</v>
-      </c>
-      <c r="O36">
+        <v>f97p50</v>
+      </c>
+      <c r="N36">
+        <v>5</v>
+      </c>
+      <c r="O36" t="s">
+        <v>336</v>
+      </c>
+      <c r="P36">
         <v>31</v>
       </c>
-      <c r="P36" t="s">
-        <v>263</v>
-      </c>
       <c r="Q36" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="37" spans="2:17">
+        <v>337</v>
+      </c>
+      <c r="R36" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="37" spans="2:18">
       <c r="B37" t="str">
         <f t="shared" si="0"/>
         <v>vs~0032</v>
       </c>
       <c r="C37" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).jAnn</v>
+        <v>d 1.5 deg OS.f97p50</v>
       </c>
       <c r="H37" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).jAnn</v>
+        <v>d 1.5 deg OS.f97p50</v>
       </c>
       <c r="I37" t="str">
         <f t="shared" si="3"/>
-        <v>c 2 deg (67%)</v>
+        <v>d 1.5 deg OS</v>
       </c>
       <c r="J37" t="str">
         <f t="shared" si="4"/>
-        <v>jAnn</v>
-      </c>
-      <c r="O37">
+        <v>f97p50</v>
+      </c>
+      <c r="N37">
+        <v>5</v>
+      </c>
+      <c r="O37" t="s">
+        <v>338</v>
+      </c>
+      <c r="P37">
         <v>32</v>
       </c>
-      <c r="P37" t="s">
-        <v>238</v>
-      </c>
       <c r="Q37" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="38" spans="2:17">
+        <v>337</v>
+      </c>
+      <c r="R37" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="38" spans="2:18">
       <c r="B38" t="str">
         <f t="shared" si="0"/>
         <v>vs~0033</v>
       </c>
       <c r="C38" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).iTS12</v>
+        <v>c 2 deg (67%).f97p50</v>
       </c>
       <c r="H38" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).iTS12</v>
+        <v>c 2 deg (67%).f97p50</v>
       </c>
       <c r="I38" t="str">
         <f t="shared" si="3"/>
@@ -5677,30 +6148,36 @@
       </c>
       <c r="J38" t="str">
         <f t="shared" si="4"/>
-        <v>iTS12</v>
-      </c>
-      <c r="O38">
+        <v>f97p50</v>
+      </c>
+      <c r="N38">
+        <v>5</v>
+      </c>
+      <c r="O38" t="s">
+        <v>339</v>
+      </c>
+      <c r="P38">
         <v>33</v>
       </c>
-      <c r="P38" t="s">
-        <v>239</v>
-      </c>
       <c r="Q38" t="s">
+        <v>337</v>
+      </c>
+      <c r="R38" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="39" spans="2:17">
+    <row r="39" spans="2:18">
       <c r="B39" t="str">
         <f t="shared" si="0"/>
         <v>vs~0034</v>
       </c>
       <c r="C39" t="str">
         <f t="shared" si="5"/>
-        <v>b 2 deg (50%).e3d</v>
+        <v>b 2 deg (50%).f97p50</v>
       </c>
       <c r="H39" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).e3d</v>
+        <v>b 2 deg (50%).f97p50</v>
       </c>
       <c r="I39" t="str">
         <f t="shared" si="3"/>
@@ -5708,154 +6185,184 @@
       </c>
       <c r="J39" t="str">
         <f t="shared" si="4"/>
-        <v>e3d</v>
-      </c>
-      <c r="O39">
+        <v>f97p50</v>
+      </c>
+      <c r="N39">
+        <v>5</v>
+      </c>
+      <c r="O39" t="s">
+        <v>340</v>
+      </c>
+      <c r="P39">
         <v>34</v>
       </c>
-      <c r="P39" t="s">
-        <v>230</v>
-      </c>
       <c r="Q39" t="s">
+        <v>337</v>
+      </c>
+      <c r="R39" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="40" spans="2:17">
+    <row r="40" spans="2:18">
       <c r="B40" t="str">
         <f t="shared" si="0"/>
         <v>vs~0035</v>
       </c>
       <c r="C40" t="str">
         <f t="shared" si="5"/>
-        <v>b 2 deg (50%).d9d</v>
+        <v>a 3 deg.f97p50</v>
       </c>
       <c r="H40" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).d9d</v>
+        <v>a 3 deg.f97p50</v>
       </c>
       <c r="I40" t="str">
         <f t="shared" si="3"/>
-        <v>b 2 deg (50%)</v>
+        <v>a 3 deg</v>
       </c>
       <c r="J40" t="str">
         <f t="shared" si="4"/>
-        <v>d9d</v>
-      </c>
-      <c r="O40">
+        <v>f97p50</v>
+      </c>
+      <c r="N40">
+        <v>5</v>
+      </c>
+      <c r="O40" t="s">
+        <v>341</v>
+      </c>
+      <c r="P40">
         <v>35</v>
       </c>
-      <c r="P40" t="s">
-        <v>231</v>
-      </c>
       <c r="Q40" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="41" spans="2:17">
+        <v>337</v>
+      </c>
+      <c r="R40" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="41" spans="2:18">
       <c r="B41" t="str">
         <f t="shared" si="0"/>
         <v>vs~0036</v>
       </c>
       <c r="C41" t="str">
         <f t="shared" ref="C41:C55" si="6">H41</f>
-        <v>b 2 deg (50%).b2w</v>
+        <v>e 1.5 deg no OS.f96p10</v>
       </c>
       <c r="H41" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).b2w</v>
+        <v>e 1.5 deg no OS.f96p10</v>
       </c>
       <c r="I41" t="str">
         <f t="shared" si="3"/>
-        <v>b 2 deg (50%)</v>
+        <v>e 1.5 deg no OS</v>
       </c>
       <c r="J41" t="str">
         <f t="shared" si="4"/>
-        <v>b2w</v>
-      </c>
-      <c r="O41">
+        <v>f96p10</v>
+      </c>
+      <c r="N41">
+        <v>5</v>
+      </c>
+      <c r="O41" t="s">
+        <v>342</v>
+      </c>
+      <c r="P41">
         <v>36</v>
       </c>
-      <c r="P41" t="s">
-        <v>232</v>
-      </c>
       <c r="Q41" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="42" spans="2:17">
+        <v>343</v>
+      </c>
+      <c r="R41" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="42" spans="2:18">
       <c r="B42" t="str">
         <f t="shared" si="0"/>
         <v>vs~0037</v>
       </c>
       <c r="C42" t="str">
         <f t="shared" si="6"/>
-        <v>b 2 deg (50%).a2w2d</v>
+        <v>d 1.5 deg OS.f96p10</v>
       </c>
       <c r="H42" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).a2w2d</v>
+        <v>d 1.5 deg OS.f96p10</v>
       </c>
       <c r="I42" t="str">
         <f t="shared" si="3"/>
-        <v>b 2 deg (50%)</v>
+        <v>d 1.5 deg OS</v>
       </c>
       <c r="J42" t="str">
         <f t="shared" si="4"/>
-        <v>a2w2d</v>
-      </c>
-      <c r="O42">
+        <v>f96p10</v>
+      </c>
+      <c r="N42">
+        <v>5</v>
+      </c>
+      <c r="O42" t="s">
+        <v>344</v>
+      </c>
+      <c r="P42">
         <v>37</v>
       </c>
-      <c r="P42" t="s">
-        <v>233</v>
-      </c>
       <c r="Q42" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="43" spans="2:17">
+        <v>343</v>
+      </c>
+      <c r="R42" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="43" spans="2:18">
       <c r="B43" t="str">
         <f t="shared" si="0"/>
         <v>vs~0038</v>
       </c>
       <c r="C43" t="str">
         <f t="shared" si="6"/>
-        <v>b 2 deg (50%).hTS12c</v>
+        <v>c 2 deg (67%).f96p10</v>
       </c>
       <c r="H43" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).hTS12c</v>
+        <v>c 2 deg (67%).f96p10</v>
       </c>
       <c r="I43" t="str">
         <f t="shared" si="3"/>
-        <v>b 2 deg (50%)</v>
+        <v>c 2 deg (67%)</v>
       </c>
       <c r="J43" t="str">
         <f t="shared" si="4"/>
-        <v>hTS12c</v>
-      </c>
-      <c r="O43">
+        <v>f96p10</v>
+      </c>
+      <c r="N43">
+        <v>5</v>
+      </c>
+      <c r="O43" t="s">
+        <v>345</v>
+      </c>
+      <c r="P43">
         <v>38</v>
       </c>
-      <c r="P43" t="s">
-        <v>234</v>
-      </c>
       <c r="Q43" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="44" spans="2:17">
+        <v>343</v>
+      </c>
+      <c r="R43" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="44" spans="2:18">
       <c r="B44" t="str">
         <f t="shared" si="0"/>
         <v>vs~0039</v>
       </c>
       <c r="C44" t="str">
         <f t="shared" si="6"/>
-        <v>b 2 deg (50%).gTS24c</v>
+        <v>b 2 deg (50%).f96p10</v>
       </c>
       <c r="H44" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).gTS24c</v>
+        <v>b 2 deg (50%).f96p10</v>
       </c>
       <c r="I44" t="str">
         <f t="shared" si="3"/>
@@ -5863,154 +6370,184 @@
       </c>
       <c r="J44" t="str">
         <f t="shared" si="4"/>
-        <v>gTS24c</v>
-      </c>
-      <c r="O44">
+        <v>f96p10</v>
+      </c>
+      <c r="N44">
+        <v>5</v>
+      </c>
+      <c r="O44" t="s">
+        <v>346</v>
+      </c>
+      <c r="P44">
         <v>39</v>
       </c>
-      <c r="P44" t="s">
-        <v>235</v>
-      </c>
       <c r="Q44" t="s">
+        <v>343</v>
+      </c>
+      <c r="R44" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="45" spans="2:17">
+    <row r="45" spans="2:18">
       <c r="B45" t="str">
         <f t="shared" si="0"/>
         <v>vs~0040</v>
       </c>
       <c r="C45" t="str">
         <f t="shared" si="6"/>
-        <v>b 2 deg (50%).fTS48c</v>
+        <v>a 3 deg.f96p10</v>
       </c>
       <c r="H45" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).fTS48c</v>
+        <v>a 3 deg.f96p10</v>
       </c>
       <c r="I45" t="str">
         <f t="shared" si="3"/>
-        <v>b 2 deg (50%)</v>
+        <v>a 3 deg</v>
       </c>
       <c r="J45" t="str">
         <f t="shared" si="4"/>
-        <v>fTS48c</v>
-      </c>
-      <c r="O45">
+        <v>f96p10</v>
+      </c>
+      <c r="N45">
+        <v>5</v>
+      </c>
+      <c r="O45" t="s">
+        <v>347</v>
+      </c>
+      <c r="P45">
         <v>40</v>
       </c>
-      <c r="P45" t="s">
-        <v>236</v>
-      </c>
       <c r="Q45" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="46" spans="2:17">
+        <v>343</v>
+      </c>
+      <c r="R45" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="46" spans="2:18">
       <c r="B46" t="str">
         <f t="shared" si="0"/>
         <v>vs~0041</v>
       </c>
       <c r="C46" t="str">
         <f t="shared" si="6"/>
-        <v>b 2 deg (50%).c15d</v>
+        <v>e 1.5 deg no OS.f96p90</v>
       </c>
       <c r="H46" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).c15d</v>
+        <v>e 1.5 deg no OS.f96p90</v>
       </c>
       <c r="I46" t="str">
         <f t="shared" si="3"/>
-        <v>b 2 deg (50%)</v>
+        <v>e 1.5 deg no OS</v>
       </c>
       <c r="J46" t="str">
         <f t="shared" si="4"/>
-        <v>c15d</v>
-      </c>
-      <c r="O46">
+        <v>f96p90</v>
+      </c>
+      <c r="N46">
+        <v>5</v>
+      </c>
+      <c r="O46" t="s">
+        <v>348</v>
+      </c>
+      <c r="P46">
         <v>41</v>
       </c>
-      <c r="P46" t="s">
-        <v>237</v>
-      </c>
       <c r="Q46" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="47" spans="2:17">
+        <v>349</v>
+      </c>
+      <c r="R46" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="47" spans="2:18">
       <c r="B47" t="str">
         <f t="shared" si="0"/>
         <v>vs~0042</v>
       </c>
       <c r="C47" t="str">
         <f t="shared" si="6"/>
-        <v>b 2 deg (50%).f1d</v>
+        <v>d 1.5 deg OS.f96p90</v>
       </c>
       <c r="H47" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).f1d</v>
+        <v>d 1.5 deg OS.f96p90</v>
       </c>
       <c r="I47" t="str">
         <f t="shared" si="3"/>
-        <v>b 2 deg (50%)</v>
+        <v>d 1.5 deg OS</v>
       </c>
       <c r="J47" t="str">
         <f t="shared" si="4"/>
-        <v>f1d</v>
-      </c>
-      <c r="O47">
+        <v>f96p90</v>
+      </c>
+      <c r="N47">
+        <v>5</v>
+      </c>
+      <c r="O47" t="s">
+        <v>350</v>
+      </c>
+      <c r="P47">
         <v>42</v>
       </c>
-      <c r="P47" t="s">
-        <v>263</v>
-      </c>
       <c r="Q47" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="48" spans="2:17">
+        <v>349</v>
+      </c>
+      <c r="R47" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="48" spans="2:18">
       <c r="B48" t="str">
         <f t="shared" si="0"/>
         <v>vs~0043</v>
       </c>
       <c r="C48" t="str">
         <f t="shared" si="6"/>
-        <v>b 2 deg (50%).jAnn</v>
+        <v>c 2 deg (67%).f96p90</v>
       </c>
       <c r="H48" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).jAnn</v>
+        <v>c 2 deg (67%).f96p90</v>
       </c>
       <c r="I48" t="str">
         <f t="shared" si="3"/>
-        <v>b 2 deg (50%)</v>
+        <v>c 2 deg (67%)</v>
       </c>
       <c r="J48" t="str">
         <f t="shared" si="4"/>
-        <v>jAnn</v>
-      </c>
-      <c r="O48">
+        <v>f96p90</v>
+      </c>
+      <c r="N48">
+        <v>5</v>
+      </c>
+      <c r="O48" t="s">
+        <v>351</v>
+      </c>
+      <c r="P48">
         <v>43</v>
       </c>
-      <c r="P48" t="s">
-        <v>238</v>
-      </c>
       <c r="Q48" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="49" spans="2:17">
+        <v>349</v>
+      </c>
+      <c r="R48" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="49" spans="2:18">
       <c r="B49" t="str">
         <f t="shared" si="0"/>
         <v>vs~0044</v>
       </c>
       <c r="C49" t="str">
         <f t="shared" si="6"/>
-        <v>b 2 deg (50%).iTS12</v>
+        <v>b 2 deg (50%).f96p90</v>
       </c>
       <c r="H49" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).iTS12</v>
+        <v>b 2 deg (50%).f96p90</v>
       </c>
       <c r="I49" t="str">
         <f t="shared" si="3"/>
@@ -6018,30 +6555,36 @@
       </c>
       <c r="J49" t="str">
         <f t="shared" si="4"/>
-        <v>iTS12</v>
-      </c>
-      <c r="O49">
+        <v>f96p90</v>
+      </c>
+      <c r="N49">
+        <v>5</v>
+      </c>
+      <c r="O49" t="s">
+        <v>352</v>
+      </c>
+      <c r="P49">
         <v>44</v>
       </c>
-      <c r="P49" t="s">
-        <v>239</v>
-      </c>
       <c r="Q49" t="s">
+        <v>349</v>
+      </c>
+      <c r="R49" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="50" spans="2:17">
+    <row r="50" spans="2:18">
       <c r="B50" t="str">
         <f t="shared" si="0"/>
         <v>vs~0045</v>
       </c>
       <c r="C50" t="str">
         <f t="shared" si="6"/>
-        <v>a 3 deg.e3d</v>
+        <v>a 3 deg.f96p90</v>
       </c>
       <c r="H50" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.e3d</v>
+        <v>a 3 deg.f96p90</v>
       </c>
       <c r="I50" t="str">
         <f t="shared" si="3"/>
@@ -6049,154 +6592,184 @@
       </c>
       <c r="J50" t="str">
         <f t="shared" si="4"/>
-        <v>e3d</v>
-      </c>
-      <c r="O50">
+        <v>f96p90</v>
+      </c>
+      <c r="N50">
+        <v>5</v>
+      </c>
+      <c r="O50" t="s">
+        <v>353</v>
+      </c>
+      <c r="P50">
         <v>45</v>
       </c>
-      <c r="P50" t="s">
-        <v>230</v>
-      </c>
       <c r="Q50" t="s">
+        <v>349</v>
+      </c>
+      <c r="R50" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="51" spans="2:17">
+    <row r="51" spans="2:18">
       <c r="B51" t="str">
         <f t="shared" si="0"/>
         <v>vs~0046</v>
       </c>
       <c r="C51" t="str">
         <f t="shared" si="6"/>
-        <v>a 3 deg.d9d</v>
+        <v>e 1.5 deg no OS.e3d</v>
       </c>
       <c r="H51" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.d9d</v>
+        <v>e 1.5 deg no OS.e3d</v>
       </c>
       <c r="I51" t="str">
         <f t="shared" si="3"/>
-        <v>a 3 deg</v>
+        <v>e 1.5 deg no OS</v>
       </c>
       <c r="J51" t="str">
         <f t="shared" si="4"/>
-        <v>d9d</v>
-      </c>
-      <c r="O51">
+        <v>e3d</v>
+      </c>
+      <c r="N51">
+        <v>5</v>
+      </c>
+      <c r="O51" t="s">
+        <v>354</v>
+      </c>
+      <c r="P51">
         <v>46</v>
       </c>
-      <c r="P51" t="s">
-        <v>231</v>
-      </c>
       <c r="Q51" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="52" spans="2:17">
+        <v>230</v>
+      </c>
+      <c r="R51" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="52" spans="2:18">
       <c r="B52" t="str">
         <f t="shared" si="0"/>
         <v>vs~0047</v>
       </c>
       <c r="C52" t="str">
         <f t="shared" si="6"/>
-        <v>a 3 deg.b2w</v>
+        <v>d 1.5 deg OS.e3d</v>
       </c>
       <c r="H52" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.b2w</v>
+        <v>d 1.5 deg OS.e3d</v>
       </c>
       <c r="I52" t="str">
         <f t="shared" si="3"/>
-        <v>a 3 deg</v>
+        <v>d 1.5 deg OS</v>
       </c>
       <c r="J52" t="str">
         <f t="shared" si="4"/>
-        <v>b2w</v>
-      </c>
-      <c r="O52">
+        <v>e3d</v>
+      </c>
+      <c r="N52">
+        <v>5</v>
+      </c>
+      <c r="O52" t="s">
+        <v>355</v>
+      </c>
+      <c r="P52">
         <v>47</v>
       </c>
-      <c r="P52" t="s">
-        <v>232</v>
-      </c>
       <c r="Q52" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="53" spans="2:17">
+        <v>230</v>
+      </c>
+      <c r="R52" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="53" spans="2:18">
       <c r="B53" t="str">
         <f t="shared" si="0"/>
         <v>vs~0048</v>
       </c>
       <c r="C53" t="str">
         <f t="shared" si="6"/>
-        <v>a 3 deg.a2w2d</v>
+        <v>c 2 deg (67%).e3d</v>
       </c>
       <c r="H53" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.a2w2d</v>
+        <v>c 2 deg (67%).e3d</v>
       </c>
       <c r="I53" t="str">
         <f t="shared" si="3"/>
-        <v>a 3 deg</v>
+        <v>c 2 deg (67%)</v>
       </c>
       <c r="J53" t="str">
         <f t="shared" si="4"/>
-        <v>a2w2d</v>
-      </c>
-      <c r="O53">
+        <v>e3d</v>
+      </c>
+      <c r="N53">
+        <v>5</v>
+      </c>
+      <c r="O53" t="s">
+        <v>356</v>
+      </c>
+      <c r="P53">
         <v>48</v>
       </c>
-      <c r="P53" t="s">
-        <v>233</v>
-      </c>
       <c r="Q53" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="54" spans="2:17">
+        <v>230</v>
+      </c>
+      <c r="R53" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="54" spans="2:18">
       <c r="B54" t="str">
         <f t="shared" si="0"/>
         <v>vs~0049</v>
       </c>
       <c r="C54" t="str">
         <f t="shared" si="6"/>
-        <v>a 3 deg.hTS12c</v>
+        <v>b 2 deg (50%).e3d</v>
       </c>
       <c r="H54" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.hTS12c</v>
+        <v>b 2 deg (50%).e3d</v>
       </c>
       <c r="I54" t="str">
         <f t="shared" si="3"/>
-        <v>a 3 deg</v>
+        <v>b 2 deg (50%)</v>
       </c>
       <c r="J54" t="str">
         <f t="shared" si="4"/>
-        <v>hTS12c</v>
-      </c>
-      <c r="O54">
+        <v>e3d</v>
+      </c>
+      <c r="N54">
+        <v>5</v>
+      </c>
+      <c r="O54" t="s">
+        <v>357</v>
+      </c>
+      <c r="P54">
         <v>49</v>
       </c>
-      <c r="P54" t="s">
-        <v>234</v>
-      </c>
       <c r="Q54" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="55" spans="2:17">
+        <v>230</v>
+      </c>
+      <c r="R54" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="55" spans="2:18">
       <c r="B55" t="str">
         <f t="shared" si="0"/>
         <v>vs~0050</v>
       </c>
       <c r="C55" t="str">
         <f t="shared" si="6"/>
-        <v>a 3 deg.gTS24c</v>
+        <v>a 3 deg.e3d</v>
       </c>
       <c r="H55" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.gTS24c</v>
+        <v>a 3 deg.e3d</v>
       </c>
       <c r="I55" t="str">
         <f t="shared" si="3"/>
@@ -6204,170 +6777,761 @@
       </c>
       <c r="J55" t="str">
         <f t="shared" si="4"/>
-        <v>gTS24c</v>
-      </c>
-      <c r="O55">
+        <v>e3d</v>
+      </c>
+      <c r="N55">
+        <v>5</v>
+      </c>
+      <c r="O55" t="s">
+        <v>358</v>
+      </c>
+      <c r="P55">
         <v>50</v>
       </c>
-      <c r="P55" t="s">
-        <v>235</v>
-      </c>
       <c r="Q55" t="s">
+        <v>230</v>
+      </c>
+      <c r="R55" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="56" spans="2:17">
+    <row r="56" spans="2:18">
       <c r="B56" t="str">
         <f t="shared" si="0"/>
         <v>vs~0051</v>
       </c>
       <c r="C56" t="str">
         <f t="shared" ref="C56:C60" si="7">H56</f>
-        <v>a 3 deg.fTS48c</v>
+        <v>e 1.5 deg no OS.d9d</v>
       </c>
       <c r="H56" t="str">
-        <f t="shared" ref="H56:H60" si="8">_xlfn.TEXTJOIN(".",TRUE,I56:J56)</f>
-        <v>a 3 deg.fTS48c</v>
+        <f t="shared" si="2"/>
+        <v>e 1.5 deg no OS.d9d</v>
       </c>
       <c r="I56" t="str">
         <f t="shared" si="3"/>
-        <v>a 3 deg</v>
+        <v>e 1.5 deg no OS</v>
       </c>
       <c r="J56" t="str">
         <f t="shared" si="4"/>
-        <v>fTS48c</v>
-      </c>
-      <c r="O56">
+        <v>d9d</v>
+      </c>
+      <c r="N56">
+        <v>5</v>
+      </c>
+      <c r="O56" t="s">
+        <v>359</v>
+      </c>
+      <c r="P56">
         <v>51</v>
       </c>
-      <c r="P56" t="s">
-        <v>236</v>
-      </c>
       <c r="Q56" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="57" spans="2:17">
+        <v>231</v>
+      </c>
+      <c r="R56" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="57" spans="2:18">
       <c r="B57" t="str">
         <f t="shared" si="0"/>
         <v>vs~0052</v>
       </c>
       <c r="C57" t="str">
         <f t="shared" si="7"/>
-        <v>a 3 deg.c15d</v>
+        <v>d 1.5 deg OS.d9d</v>
       </c>
       <c r="H57" t="str">
-        <f t="shared" si="8"/>
-        <v>a 3 deg.c15d</v>
+        <f t="shared" si="2"/>
+        <v>d 1.5 deg OS.d9d</v>
       </c>
       <c r="I57" t="str">
         <f t="shared" si="3"/>
-        <v>a 3 deg</v>
+        <v>d 1.5 deg OS</v>
       </c>
       <c r="J57" t="str">
         <f t="shared" si="4"/>
-        <v>c15d</v>
-      </c>
-      <c r="O57">
+        <v>d9d</v>
+      </c>
+      <c r="N57">
+        <v>5</v>
+      </c>
+      <c r="O57" t="s">
+        <v>360</v>
+      </c>
+      <c r="P57">
         <v>52</v>
       </c>
-      <c r="P57" t="s">
-        <v>237</v>
-      </c>
       <c r="Q57" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="58" spans="2:17">
+        <v>231</v>
+      </c>
+      <c r="R57" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="58" spans="2:18">
       <c r="B58" t="str">
         <f t="shared" si="0"/>
         <v>vs~0053</v>
       </c>
       <c r="C58" t="str">
         <f t="shared" si="7"/>
-        <v>a 3 deg.f1d</v>
+        <v>c 2 deg (67%).d9d</v>
       </c>
       <c r="H58" t="str">
-        <f t="shared" si="8"/>
-        <v>a 3 deg.f1d</v>
+        <f t="shared" si="2"/>
+        <v>c 2 deg (67%).d9d</v>
       </c>
       <c r="I58" t="str">
         <f t="shared" si="3"/>
-        <v>a 3 deg</v>
+        <v>c 2 deg (67%)</v>
       </c>
       <c r="J58" t="str">
         <f t="shared" si="4"/>
-        <v>f1d</v>
-      </c>
-      <c r="O58">
+        <v>d9d</v>
+      </c>
+      <c r="N58">
+        <v>5</v>
+      </c>
+      <c r="O58" t="s">
+        <v>361</v>
+      </c>
+      <c r="P58">
         <v>53</v>
       </c>
-      <c r="P58" t="s">
-        <v>263</v>
-      </c>
       <c r="Q58" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="59" spans="2:17">
+        <v>231</v>
+      </c>
+      <c r="R58" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="59" spans="2:18">
       <c r="B59" t="str">
         <f t="shared" si="0"/>
         <v>vs~0054</v>
       </c>
       <c r="C59" t="str">
         <f t="shared" si="7"/>
-        <v>a 3 deg.jAnn</v>
+        <v>b 2 deg (50%).d9d</v>
       </c>
       <c r="H59" t="str">
-        <f t="shared" si="8"/>
-        <v>a 3 deg.jAnn</v>
+        <f t="shared" si="2"/>
+        <v>b 2 deg (50%).d9d</v>
       </c>
       <c r="I59" t="str">
         <f t="shared" si="3"/>
-        <v>a 3 deg</v>
+        <v>b 2 deg (50%)</v>
       </c>
       <c r="J59" t="str">
         <f t="shared" si="4"/>
-        <v>jAnn</v>
-      </c>
-      <c r="O59">
+        <v>d9d</v>
+      </c>
+      <c r="N59">
+        <v>5</v>
+      </c>
+      <c r="O59" t="s">
+        <v>362</v>
+      </c>
+      <c r="P59">
         <v>54</v>
       </c>
-      <c r="P59" t="s">
-        <v>238</v>
-      </c>
       <c r="Q59" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="60" spans="2:17">
+        <v>231</v>
+      </c>
+      <c r="R59" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="60" spans="2:18">
       <c r="B60" t="str">
         <f t="shared" si="0"/>
         <v>vs~0055</v>
       </c>
       <c r="C60" t="str">
         <f t="shared" si="7"/>
-        <v>a 3 deg.iTS12</v>
+        <v>a 3 deg.d9d</v>
       </c>
       <c r="H60" t="str">
+        <f t="shared" si="2"/>
+        <v>a 3 deg.d9d</v>
+      </c>
+      <c r="I60" t="str">
+        <f t="shared" si="3"/>
+        <v>a 3 deg</v>
+      </c>
+      <c r="J60" t="str">
+        <f t="shared" si="4"/>
+        <v>d9d</v>
+      </c>
+      <c r="N60">
+        <v>5</v>
+      </c>
+      <c r="O60" t="s">
+        <v>363</v>
+      </c>
+      <c r="P60">
+        <v>55</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>231</v>
+      </c>
+      <c r="R60" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="61" spans="2:18">
+      <c r="B61" t="str">
+        <f t="shared" ref="B61:B75" si="8">"vs~"&amp;TEXT(P61,"0000")</f>
+        <v>vs~0056</v>
+      </c>
+      <c r="C61" t="str">
+        <f t="shared" ref="C61:C75" si="9">H61</f>
+        <v>e 1.5 deg no OS.c15d</v>
+      </c>
+      <c r="H61" t="str">
+        <f t="shared" ref="H61:H75" si="10">_xlfn.TEXTJOIN(".",TRUE,I61:J61)</f>
+        <v>e 1.5 deg no OS.c15d</v>
+      </c>
+      <c r="I61" t="str">
+        <f t="shared" ref="I61:I75" si="11">VLOOKUP(R61,$W$6:$X$12,2,FALSE)</f>
+        <v>e 1.5 deg no OS</v>
+      </c>
+      <c r="J61" t="str">
+        <f t="shared" ref="J61:J75" si="12">VLOOKUP(Q61,$T$6:$U$20,2,FALSE)</f>
+        <v>c15d</v>
+      </c>
+      <c r="N61">
+        <v>5</v>
+      </c>
+      <c r="O61" t="s">
+        <v>364</v>
+      </c>
+      <c r="P61">
+        <v>56</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>237</v>
+      </c>
+      <c r="R61" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="62" spans="2:18">
+      <c r="B62" t="str">
         <f t="shared" si="8"/>
-        <v>a 3 deg.iTS12</v>
-      </c>
-      <c r="I60" t="str">
-        <f t="shared" si="3"/>
+        <v>vs~0057</v>
+      </c>
+      <c r="C62" t="str">
+        <f t="shared" si="9"/>
+        <v>d 1.5 deg OS.c15d</v>
+      </c>
+      <c r="H62" t="str">
+        <f t="shared" si="10"/>
+        <v>d 1.5 deg OS.c15d</v>
+      </c>
+      <c r="I62" t="str">
+        <f t="shared" si="11"/>
+        <v>d 1.5 deg OS</v>
+      </c>
+      <c r="J62" t="str">
+        <f t="shared" si="12"/>
+        <v>c15d</v>
+      </c>
+      <c r="N62">
+        <v>5</v>
+      </c>
+      <c r="O62" t="s">
+        <v>365</v>
+      </c>
+      <c r="P62">
+        <v>57</v>
+      </c>
+      <c r="Q62" t="s">
+        <v>237</v>
+      </c>
+      <c r="R62" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="63" spans="2:18">
+      <c r="B63" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0058</v>
+      </c>
+      <c r="C63" t="str">
+        <f t="shared" si="9"/>
+        <v>c 2 deg (67%).c15d</v>
+      </c>
+      <c r="H63" t="str">
+        <f t="shared" si="10"/>
+        <v>c 2 deg (67%).c15d</v>
+      </c>
+      <c r="I63" t="str">
+        <f t="shared" si="11"/>
+        <v>c 2 deg (67%)</v>
+      </c>
+      <c r="J63" t="str">
+        <f t="shared" si="12"/>
+        <v>c15d</v>
+      </c>
+      <c r="N63">
+        <v>5</v>
+      </c>
+      <c r="O63" t="s">
+        <v>366</v>
+      </c>
+      <c r="P63">
+        <v>58</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>237</v>
+      </c>
+      <c r="R63" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="64" spans="2:18">
+      <c r="B64" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0059</v>
+      </c>
+      <c r="C64" t="str">
+        <f t="shared" si="9"/>
+        <v>b 2 deg (50%).c15d</v>
+      </c>
+      <c r="H64" t="str">
+        <f t="shared" si="10"/>
+        <v>b 2 deg (50%).c15d</v>
+      </c>
+      <c r="I64" t="str">
+        <f t="shared" si="11"/>
+        <v>b 2 deg (50%)</v>
+      </c>
+      <c r="J64" t="str">
+        <f t="shared" si="12"/>
+        <v>c15d</v>
+      </c>
+      <c r="N64">
+        <v>5</v>
+      </c>
+      <c r="O64" t="s">
+        <v>367</v>
+      </c>
+      <c r="P64">
+        <v>59</v>
+      </c>
+      <c r="Q64" t="s">
+        <v>237</v>
+      </c>
+      <c r="R64" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="65" spans="2:18">
+      <c r="B65" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0060</v>
+      </c>
+      <c r="C65" t="str">
+        <f t="shared" si="9"/>
+        <v>a 3 deg.c15d</v>
+      </c>
+      <c r="H65" t="str">
+        <f t="shared" si="10"/>
+        <v>a 3 deg.c15d</v>
+      </c>
+      <c r="I65" t="str">
+        <f t="shared" si="11"/>
         <v>a 3 deg</v>
       </c>
-      <c r="J60" t="str">
-        <f t="shared" si="4"/>
-        <v>iTS12</v>
-      </c>
-      <c r="O60">
-        <v>55</v>
-      </c>
-      <c r="P60" t="s">
-        <v>239</v>
-      </c>
-      <c r="Q60" t="s">
+      <c r="J65" t="str">
+        <f t="shared" si="12"/>
+        <v>c15d</v>
+      </c>
+      <c r="N65">
+        <v>5</v>
+      </c>
+      <c r="O65" t="s">
+        <v>368</v>
+      </c>
+      <c r="P65">
+        <v>60</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>237</v>
+      </c>
+      <c r="R65" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="66" spans="2:18">
+      <c r="B66" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0061</v>
+      </c>
+      <c r="C66" t="str">
+        <f t="shared" si="9"/>
+        <v>e 1.5 deg no OS.b2w</v>
+      </c>
+      <c r="H66" t="str">
+        <f t="shared" si="10"/>
+        <v>e 1.5 deg no OS.b2w</v>
+      </c>
+      <c r="I66" t="str">
+        <f t="shared" si="11"/>
+        <v>e 1.5 deg no OS</v>
+      </c>
+      <c r="J66" t="str">
+        <f t="shared" si="12"/>
+        <v>b2w</v>
+      </c>
+      <c r="N66">
+        <v>5</v>
+      </c>
+      <c r="O66" t="s">
+        <v>369</v>
+      </c>
+      <c r="P66">
+        <v>61</v>
+      </c>
+      <c r="Q66" t="s">
+        <v>232</v>
+      </c>
+      <c r="R66" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="67" spans="2:18">
+      <c r="B67" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0062</v>
+      </c>
+      <c r="C67" t="str">
+        <f t="shared" si="9"/>
+        <v>d 1.5 deg OS.b2w</v>
+      </c>
+      <c r="H67" t="str">
+        <f t="shared" si="10"/>
+        <v>d 1.5 deg OS.b2w</v>
+      </c>
+      <c r="I67" t="str">
+        <f t="shared" si="11"/>
+        <v>d 1.5 deg OS</v>
+      </c>
+      <c r="J67" t="str">
+        <f t="shared" si="12"/>
+        <v>b2w</v>
+      </c>
+      <c r="N67">
+        <v>5</v>
+      </c>
+      <c r="O67" t="s">
+        <v>370</v>
+      </c>
+      <c r="P67">
+        <v>62</v>
+      </c>
+      <c r="Q67" t="s">
+        <v>232</v>
+      </c>
+      <c r="R67" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="68" spans="2:18">
+      <c r="B68" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0063</v>
+      </c>
+      <c r="C68" t="str">
+        <f t="shared" si="9"/>
+        <v>c 2 deg (67%).b2w</v>
+      </c>
+      <c r="H68" t="str">
+        <f t="shared" si="10"/>
+        <v>c 2 deg (67%).b2w</v>
+      </c>
+      <c r="I68" t="str">
+        <f t="shared" si="11"/>
+        <v>c 2 deg (67%)</v>
+      </c>
+      <c r="J68" t="str">
+        <f t="shared" si="12"/>
+        <v>b2w</v>
+      </c>
+      <c r="N68">
+        <v>5</v>
+      </c>
+      <c r="O68" t="s">
+        <v>371</v>
+      </c>
+      <c r="P68">
+        <v>63</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>232</v>
+      </c>
+      <c r="R68" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="69" spans="2:18">
+      <c r="B69" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0064</v>
+      </c>
+      <c r="C69" t="str">
+        <f t="shared" si="9"/>
+        <v>b 2 deg (50%).b2w</v>
+      </c>
+      <c r="H69" t="str">
+        <f t="shared" si="10"/>
+        <v>b 2 deg (50%).b2w</v>
+      </c>
+      <c r="I69" t="str">
+        <f t="shared" si="11"/>
+        <v>b 2 deg (50%)</v>
+      </c>
+      <c r="J69" t="str">
+        <f t="shared" si="12"/>
+        <v>b2w</v>
+      </c>
+      <c r="N69">
+        <v>5</v>
+      </c>
+      <c r="O69" t="s">
+        <v>372</v>
+      </c>
+      <c r="P69">
+        <v>64</v>
+      </c>
+      <c r="Q69" t="s">
+        <v>232</v>
+      </c>
+      <c r="R69" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="70" spans="2:18">
+      <c r="B70" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0065</v>
+      </c>
+      <c r="C70" t="str">
+        <f t="shared" si="9"/>
+        <v>a 3 deg.b2w</v>
+      </c>
+      <c r="H70" t="str">
+        <f t="shared" si="10"/>
+        <v>a 3 deg.b2w</v>
+      </c>
+      <c r="I70" t="str">
+        <f t="shared" si="11"/>
+        <v>a 3 deg</v>
+      </c>
+      <c r="J70" t="str">
+        <f t="shared" si="12"/>
+        <v>b2w</v>
+      </c>
+      <c r="N70">
+        <v>5</v>
+      </c>
+      <c r="O70" t="s">
+        <v>373</v>
+      </c>
+      <c r="P70">
+        <v>65</v>
+      </c>
+      <c r="Q70" t="s">
+        <v>232</v>
+      </c>
+      <c r="R70" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="71" spans="2:18">
+      <c r="B71" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0066</v>
+      </c>
+      <c r="C71" t="str">
+        <f t="shared" si="9"/>
+        <v>e 1.5 deg no OS.a2w2d</v>
+      </c>
+      <c r="H71" t="str">
+        <f t="shared" si="10"/>
+        <v>e 1.5 deg no OS.a2w2d</v>
+      </c>
+      <c r="I71" t="str">
+        <f t="shared" si="11"/>
+        <v>e 1.5 deg no OS</v>
+      </c>
+      <c r="J71" t="str">
+        <f t="shared" si="12"/>
+        <v>a2w2d</v>
+      </c>
+      <c r="N71">
+        <v>5</v>
+      </c>
+      <c r="O71" t="s">
+        <v>374</v>
+      </c>
+      <c r="P71">
+        <v>66</v>
+      </c>
+      <c r="Q71" t="s">
+        <v>233</v>
+      </c>
+      <c r="R71" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="72" spans="2:18">
+      <c r="B72" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0067</v>
+      </c>
+      <c r="C72" t="str">
+        <f t="shared" si="9"/>
+        <v>d 1.5 deg OS.a2w2d</v>
+      </c>
+      <c r="H72" t="str">
+        <f t="shared" si="10"/>
+        <v>d 1.5 deg OS.a2w2d</v>
+      </c>
+      <c r="I72" t="str">
+        <f t="shared" si="11"/>
+        <v>d 1.5 deg OS</v>
+      </c>
+      <c r="J72" t="str">
+        <f t="shared" si="12"/>
+        <v>a2w2d</v>
+      </c>
+      <c r="N72">
+        <v>5</v>
+      </c>
+      <c r="O72" t="s">
+        <v>375</v>
+      </c>
+      <c r="P72">
+        <v>67</v>
+      </c>
+      <c r="Q72" t="s">
+        <v>233</v>
+      </c>
+      <c r="R72" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="73" spans="2:18">
+      <c r="B73" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0068</v>
+      </c>
+      <c r="C73" t="str">
+        <f t="shared" si="9"/>
+        <v>c 2 deg (67%).a2w2d</v>
+      </c>
+      <c r="H73" t="str">
+        <f t="shared" si="10"/>
+        <v>c 2 deg (67%).a2w2d</v>
+      </c>
+      <c r="I73" t="str">
+        <f t="shared" si="11"/>
+        <v>c 2 deg (67%)</v>
+      </c>
+      <c r="J73" t="str">
+        <f t="shared" si="12"/>
+        <v>a2w2d</v>
+      </c>
+      <c r="N73">
+        <v>5</v>
+      </c>
+      <c r="O73" t="s">
+        <v>376</v>
+      </c>
+      <c r="P73">
+        <v>68</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>233</v>
+      </c>
+      <c r="R73" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="74" spans="2:18">
+      <c r="B74" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0069</v>
+      </c>
+      <c r="C74" t="str">
+        <f t="shared" si="9"/>
+        <v>b 2 deg (50%).a2w2d</v>
+      </c>
+      <c r="H74" t="str">
+        <f t="shared" si="10"/>
+        <v>b 2 deg (50%).a2w2d</v>
+      </c>
+      <c r="I74" t="str">
+        <f t="shared" si="11"/>
+        <v>b 2 deg (50%)</v>
+      </c>
+      <c r="J74" t="str">
+        <f t="shared" si="12"/>
+        <v>a2w2d</v>
+      </c>
+      <c r="N74">
+        <v>5</v>
+      </c>
+      <c r="O74" t="s">
+        <v>377</v>
+      </c>
+      <c r="P74">
+        <v>69</v>
+      </c>
+      <c r="Q74" t="s">
+        <v>233</v>
+      </c>
+      <c r="R74" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="75" spans="2:18">
+      <c r="B75" t="str">
+        <f t="shared" si="8"/>
+        <v>vs~0070</v>
+      </c>
+      <c r="C75" t="str">
+        <f t="shared" si="9"/>
+        <v>a 3 deg.a2w2d</v>
+      </c>
+      <c r="H75" t="str">
+        <f t="shared" si="10"/>
+        <v>a 3 deg.a2w2d</v>
+      </c>
+      <c r="I75" t="str">
+        <f t="shared" si="11"/>
+        <v>a 3 deg</v>
+      </c>
+      <c r="J75" t="str">
+        <f t="shared" si="12"/>
+        <v>a2w2d</v>
+      </c>
+      <c r="N75">
+        <v>5</v>
+      </c>
+      <c r="O75" t="s">
+        <v>378</v>
+      </c>
+      <c r="P75">
+        <v>70</v>
+      </c>
+      <c r="Q75" t="s">
+        <v>233</v>
+      </c>
+      <c r="R75" t="s">
         <v>289</v>
       </c>
     </row>
@@ -6812,7 +7976,7 @@
   <sheetData>
     <row r="3" spans="1:19" ht="17.25" thickBot="1">
       <c r="A3" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="15" thickTop="1" thickBot="1">

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-17 16:29
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_DEU/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBFA3B6F-77C9-4026-A7F7-2B3175ECC1C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3BCA134-6F6E-46C7-B2D4-F78ECE5CD6C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -867,9 +867,6 @@
     <t>ar6_r10</t>
   </si>
   <si>
-    <t>ELC,ELC_???-???*,e[_]*</t>
-  </si>
-  <si>
     <t>*ccs</t>
   </si>
   <si>
@@ -1239,13 +1236,16 @@
     <t>g64</t>
   </si>
   <si>
-    <t>f97p50</t>
-  </si>
-  <si>
     <t>f96p10</t>
   </si>
   <si>
     <t>f96p90</t>
+  </si>
+  <si>
+    <t>f96p50</t>
+  </si>
+  <si>
+    <t>ELC,ELC_???[_]???*,e[_]*</t>
   </si>
 </sst>
 </file>
@@ -2311,10 +2311,10 @@
         <v>11</v>
       </c>
       <c r="T16" t="s">
+        <v>262</v>
+      </c>
+      <c r="U16" t="s">
         <v>263</v>
-      </c>
-      <c r="U16" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="17" spans="1:17">
@@ -4427,7 +4427,7 @@
         <v>69</v>
       </c>
       <c r="B50" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C50" t="s">
         <v>132</v>
@@ -4441,7 +4441,7 @@
         <v>69</v>
       </c>
       <c r="B51" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C51" t="s">
         <v>133</v>
@@ -4773,7 +4773,7 @@
         <v>63</v>
       </c>
       <c r="O4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5" spans="2:24">
@@ -4801,19 +4801,19 @@
         <v>sg_timeslice</v>
       </c>
       <c r="N5" t="s">
+        <v>296</v>
+      </c>
+      <c r="O5" t="s">
         <v>297</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>298</v>
-      </c>
-      <c r="P5" t="s">
-        <v>299</v>
       </c>
       <c r="Q5" t="s">
         <v>124</v>
       </c>
       <c r="R5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="6" spans="2:24">
@@ -4844,7 +4844,7 @@
         <v>5</v>
       </c>
       <c r="O6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="P6">
         <v>1</v>
@@ -4853,16 +4853,16 @@
         <v>238</v>
       </c>
       <c r="R6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="T6" t="s">
         <v>238</v>
       </c>
       <c r="U6" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="W6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="X6" t="s">
         <v>258</v>
@@ -4896,7 +4896,7 @@
         <v>5</v>
       </c>
       <c r="O7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="P7">
         <v>2</v>
@@ -4905,16 +4905,16 @@
         <v>238</v>
       </c>
       <c r="R7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="T7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="U7" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="W7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="X7" t="s">
         <v>257</v>
@@ -4948,7 +4948,7 @@
         <v>5</v>
       </c>
       <c r="O8" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="P8">
         <v>3</v>
@@ -4957,16 +4957,16 @@
         <v>238</v>
       </c>
       <c r="R8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="T8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="U8" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="W8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="X8" t="s">
         <v>256</v>
@@ -5000,7 +5000,7 @@
         <v>5</v>
       </c>
       <c r="O9" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="P9">
         <v>4</v>
@@ -5009,16 +5009,16 @@
         <v>238</v>
       </c>
       <c r="R9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="T9" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="U9" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="W9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="X9" t="s">
         <v>255</v>
@@ -5052,7 +5052,7 @@
         <v>5</v>
       </c>
       <c r="O10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="P10">
         <v>5</v>
@@ -5061,16 +5061,16 @@
         <v>238</v>
       </c>
       <c r="R10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="T10" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="U10" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="W10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="X10" t="s">
         <v>259</v>
@@ -5101,22 +5101,22 @@
         <v>5</v>
       </c>
       <c r="O11" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="P11">
         <v>6</v>
       </c>
       <c r="Q11" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="T11" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="U11" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="12" spans="2:24">
@@ -5144,22 +5144,22 @@
         <v>5</v>
       </c>
       <c r="O12" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="P12">
         <v>7</v>
       </c>
       <c r="Q12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R12" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="T12" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="U12" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="13" spans="2:24">
@@ -5187,22 +5187,22 @@
         <v>5</v>
       </c>
       <c r="O13" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="P13">
         <v>8</v>
       </c>
       <c r="Q13" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="T13" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="U13" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="14" spans="2:24">
@@ -5230,22 +5230,22 @@
         <v>5</v>
       </c>
       <c r="O14" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="P14">
         <v>9</v>
       </c>
       <c r="Q14" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R14" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="T14" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="U14" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="15" spans="2:24">
@@ -5273,16 +5273,16 @@
         <v>5</v>
       </c>
       <c r="O15" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="P15">
         <v>10</v>
       </c>
       <c r="Q15" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="T15" t="s">
         <v>230</v>
@@ -5316,16 +5316,16 @@
         <v>5</v>
       </c>
       <c r="O16" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="P16">
         <v>11</v>
       </c>
       <c r="Q16" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="T16" t="s">
         <v>231</v>
@@ -5359,16 +5359,16 @@
         <v>5</v>
       </c>
       <c r="O17" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="P17">
         <v>12</v>
       </c>
       <c r="Q17" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R17" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="T17" t="s">
         <v>237</v>
@@ -5402,16 +5402,16 @@
         <v>5</v>
       </c>
       <c r="O18" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="P18">
         <v>13</v>
       </c>
       <c r="Q18" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R18" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="T18" t="s">
         <v>232</v>
@@ -5445,16 +5445,16 @@
         <v>5</v>
       </c>
       <c r="O19" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="P19">
         <v>14</v>
       </c>
       <c r="Q19" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R19" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="T19" t="s">
         <v>233</v>
@@ -5488,16 +5488,16 @@
         <v>5</v>
       </c>
       <c r="O20" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="P20">
         <v>15</v>
       </c>
       <c r="Q20" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R20" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="21" spans="2:21">
@@ -5525,16 +5525,16 @@
         <v>5</v>
       </c>
       <c r="O21" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="P21">
         <v>16</v>
       </c>
       <c r="Q21" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R21" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="22" spans="2:21">
@@ -5562,16 +5562,16 @@
         <v>5</v>
       </c>
       <c r="O22" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="P22">
         <v>17</v>
       </c>
       <c r="Q22" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="23" spans="2:21">
@@ -5599,16 +5599,16 @@
         <v>5</v>
       </c>
       <c r="O23" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="P23">
         <v>18</v>
       </c>
       <c r="Q23" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R23" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="24" spans="2:21">
@@ -5636,16 +5636,16 @@
         <v>5</v>
       </c>
       <c r="O24" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="P24">
         <v>19</v>
       </c>
       <c r="Q24" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R24" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="25" spans="2:21">
@@ -5673,16 +5673,16 @@
         <v>5</v>
       </c>
       <c r="O25" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="P25">
         <v>20</v>
       </c>
       <c r="Q25" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R25" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="26" spans="2:21">
@@ -5710,16 +5710,16 @@
         <v>5</v>
       </c>
       <c r="O26" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="P26">
         <v>21</v>
       </c>
       <c r="Q26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R26" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="27" spans="2:21">
@@ -5747,16 +5747,16 @@
         <v>5</v>
       </c>
       <c r="O27" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="P27">
         <v>22</v>
       </c>
       <c r="Q27" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R27" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="28" spans="2:21">
@@ -5784,16 +5784,16 @@
         <v>5</v>
       </c>
       <c r="O28" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="P28">
         <v>23</v>
       </c>
       <c r="Q28" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R28" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29" spans="2:21">
@@ -5821,16 +5821,16 @@
         <v>5</v>
       </c>
       <c r="O29" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="P29">
         <v>24</v>
       </c>
       <c r="Q29" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R29" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="30" spans="2:21">
@@ -5858,16 +5858,16 @@
         <v>5</v>
       </c>
       <c r="O30" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P30">
         <v>25</v>
       </c>
       <c r="Q30" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R30" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="31" spans="2:21">
@@ -5895,16 +5895,16 @@
         <v>5</v>
       </c>
       <c r="O31" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="P31">
         <v>26</v>
       </c>
       <c r="Q31" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R31" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="32" spans="2:21">
@@ -5932,16 +5932,16 @@
         <v>5</v>
       </c>
       <c r="O32" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="P32">
         <v>27</v>
       </c>
       <c r="Q32" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R32" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="33" spans="2:18">
@@ -5969,16 +5969,16 @@
         <v>5</v>
       </c>
       <c r="O33" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="P33">
         <v>28</v>
       </c>
       <c r="Q33" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R33" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="34" spans="2:18">
@@ -6006,16 +6006,16 @@
         <v>5</v>
       </c>
       <c r="O34" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="P34">
         <v>29</v>
       </c>
       <c r="Q34" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R34" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="35" spans="2:18">
@@ -6043,16 +6043,16 @@
         <v>5</v>
       </c>
       <c r="O35" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="P35">
         <v>30</v>
       </c>
       <c r="Q35" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R35" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="36" spans="2:18">
@@ -6062,11 +6062,11 @@
       </c>
       <c r="C36" t="str">
         <f t="shared" si="5"/>
-        <v>e 1.5 deg no OS.f97p50</v>
+        <v>e 1.5 deg no OS.f96p50</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.f97p50</v>
+        <v>e 1.5 deg no OS.f96p50</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="3"/>
@@ -6074,22 +6074,22 @@
       </c>
       <c r="J36" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N36">
         <v>5</v>
       </c>
       <c r="O36" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="P36">
         <v>31</v>
       </c>
       <c r="Q36" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R36" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="37" spans="2:18">
@@ -6099,11 +6099,11 @@
       </c>
       <c r="C37" t="str">
         <f t="shared" si="5"/>
-        <v>d 1.5 deg OS.f97p50</v>
+        <v>d 1.5 deg OS.f96p50</v>
       </c>
       <c r="H37" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.f97p50</v>
+        <v>d 1.5 deg OS.f96p50</v>
       </c>
       <c r="I37" t="str">
         <f t="shared" si="3"/>
@@ -6111,22 +6111,22 @@
       </c>
       <c r="J37" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N37">
         <v>5</v>
       </c>
       <c r="O37" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="P37">
         <v>32</v>
       </c>
       <c r="Q37" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R37" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="38" spans="2:18">
@@ -6136,11 +6136,11 @@
       </c>
       <c r="C38" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).f97p50</v>
+        <v>c 2 deg (67%).f96p50</v>
       </c>
       <c r="H38" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).f97p50</v>
+        <v>c 2 deg (67%).f96p50</v>
       </c>
       <c r="I38" t="str">
         <f t="shared" si="3"/>
@@ -6148,22 +6148,22 @@
       </c>
       <c r="J38" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N38">
         <v>5</v>
       </c>
       <c r="O38" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="P38">
         <v>33</v>
       </c>
       <c r="Q38" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R38" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="39" spans="2:18">
@@ -6173,11 +6173,11 @@
       </c>
       <c r="C39" t="str">
         <f t="shared" si="5"/>
-        <v>b 2 deg (50%).f97p50</v>
+        <v>b 2 deg (50%).f96p50</v>
       </c>
       <c r="H39" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).f97p50</v>
+        <v>b 2 deg (50%).f96p50</v>
       </c>
       <c r="I39" t="str">
         <f t="shared" si="3"/>
@@ -6185,22 +6185,22 @@
       </c>
       <c r="J39" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N39">
         <v>5</v>
       </c>
       <c r="O39" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="P39">
         <v>34</v>
       </c>
       <c r="Q39" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R39" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="40" spans="2:18">
@@ -6210,11 +6210,11 @@
       </c>
       <c r="C40" t="str">
         <f t="shared" si="5"/>
-        <v>a 3 deg.f97p50</v>
+        <v>a 3 deg.f96p50</v>
       </c>
       <c r="H40" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.f97p50</v>
+        <v>a 3 deg.f96p50</v>
       </c>
       <c r="I40" t="str">
         <f t="shared" si="3"/>
@@ -6222,22 +6222,22 @@
       </c>
       <c r="J40" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N40">
         <v>5</v>
       </c>
       <c r="O40" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="P40">
         <v>35</v>
       </c>
       <c r="Q40" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R40" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="41" spans="2:18">
@@ -6265,16 +6265,16 @@
         <v>5</v>
       </c>
       <c r="O41" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="P41">
         <v>36</v>
       </c>
       <c r="Q41" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R41" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="42" spans="2:18">
@@ -6302,16 +6302,16 @@
         <v>5</v>
       </c>
       <c r="O42" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="P42">
         <v>37</v>
       </c>
       <c r="Q42" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R42" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="43" spans="2:18">
@@ -6339,16 +6339,16 @@
         <v>5</v>
       </c>
       <c r="O43" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="P43">
         <v>38</v>
       </c>
       <c r="Q43" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R43" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="44" spans="2:18">
@@ -6376,16 +6376,16 @@
         <v>5</v>
       </c>
       <c r="O44" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="P44">
         <v>39</v>
       </c>
       <c r="Q44" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R44" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="45" spans="2:18">
@@ -6413,16 +6413,16 @@
         <v>5</v>
       </c>
       <c r="O45" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="P45">
         <v>40</v>
       </c>
       <c r="Q45" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R45" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="46" spans="2:18">
@@ -6450,16 +6450,16 @@
         <v>5</v>
       </c>
       <c r="O46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="P46">
         <v>41</v>
       </c>
       <c r="Q46" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R46" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="47" spans="2:18">
@@ -6487,16 +6487,16 @@
         <v>5</v>
       </c>
       <c r="O47" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="P47">
         <v>42</v>
       </c>
       <c r="Q47" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R47" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="48" spans="2:18">
@@ -6524,16 +6524,16 @@
         <v>5</v>
       </c>
       <c r="O48" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="P48">
         <v>43</v>
       </c>
       <c r="Q48" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R48" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="49" spans="2:18">
@@ -6561,16 +6561,16 @@
         <v>5</v>
       </c>
       <c r="O49" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="P49">
         <v>44</v>
       </c>
       <c r="Q49" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R49" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="50" spans="2:18">
@@ -6598,16 +6598,16 @@
         <v>5</v>
       </c>
       <c r="O50" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="P50">
         <v>45</v>
       </c>
       <c r="Q50" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R50" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="51" spans="2:18">
@@ -6635,7 +6635,7 @@
         <v>5</v>
       </c>
       <c r="O51" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="P51">
         <v>46</v>
@@ -6644,7 +6644,7 @@
         <v>230</v>
       </c>
       <c r="R51" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="52" spans="2:18">
@@ -6672,7 +6672,7 @@
         <v>5</v>
       </c>
       <c r="O52" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="P52">
         <v>47</v>
@@ -6681,7 +6681,7 @@
         <v>230</v>
       </c>
       <c r="R52" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="53" spans="2:18">
@@ -6709,7 +6709,7 @@
         <v>5</v>
       </c>
       <c r="O53" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="P53">
         <v>48</v>
@@ -6718,7 +6718,7 @@
         <v>230</v>
       </c>
       <c r="R53" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="54" spans="2:18">
@@ -6746,7 +6746,7 @@
         <v>5</v>
       </c>
       <c r="O54" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="P54">
         <v>49</v>
@@ -6755,7 +6755,7 @@
         <v>230</v>
       </c>
       <c r="R54" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="55" spans="2:18">
@@ -6783,7 +6783,7 @@
         <v>5</v>
       </c>
       <c r="O55" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="P55">
         <v>50</v>
@@ -6792,7 +6792,7 @@
         <v>230</v>
       </c>
       <c r="R55" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="56" spans="2:18">
@@ -6820,7 +6820,7 @@
         <v>5</v>
       </c>
       <c r="O56" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="P56">
         <v>51</v>
@@ -6829,7 +6829,7 @@
         <v>231</v>
       </c>
       <c r="R56" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="57" spans="2:18">
@@ -6857,7 +6857,7 @@
         <v>5</v>
       </c>
       <c r="O57" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="P57">
         <v>52</v>
@@ -6866,7 +6866,7 @@
         <v>231</v>
       </c>
       <c r="R57" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="58" spans="2:18">
@@ -6894,7 +6894,7 @@
         <v>5</v>
       </c>
       <c r="O58" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="P58">
         <v>53</v>
@@ -6903,7 +6903,7 @@
         <v>231</v>
       </c>
       <c r="R58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="59" spans="2:18">
@@ -6931,7 +6931,7 @@
         <v>5</v>
       </c>
       <c r="O59" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="P59">
         <v>54</v>
@@ -6940,7 +6940,7 @@
         <v>231</v>
       </c>
       <c r="R59" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="60" spans="2:18">
@@ -6968,7 +6968,7 @@
         <v>5</v>
       </c>
       <c r="O60" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="P60">
         <v>55</v>
@@ -6977,7 +6977,7 @@
         <v>231</v>
       </c>
       <c r="R60" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="61" spans="2:18">
@@ -7005,7 +7005,7 @@
         <v>5</v>
       </c>
       <c r="O61" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="P61">
         <v>56</v>
@@ -7014,7 +7014,7 @@
         <v>237</v>
       </c>
       <c r="R61" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="62" spans="2:18">
@@ -7042,7 +7042,7 @@
         <v>5</v>
       </c>
       <c r="O62" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="P62">
         <v>57</v>
@@ -7051,7 +7051,7 @@
         <v>237</v>
       </c>
       <c r="R62" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="63" spans="2:18">
@@ -7079,7 +7079,7 @@
         <v>5</v>
       </c>
       <c r="O63" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="P63">
         <v>58</v>
@@ -7088,7 +7088,7 @@
         <v>237</v>
       </c>
       <c r="R63" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="64" spans="2:18">
@@ -7116,7 +7116,7 @@
         <v>5</v>
       </c>
       <c r="O64" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="P64">
         <v>59</v>
@@ -7125,7 +7125,7 @@
         <v>237</v>
       </c>
       <c r="R64" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="65" spans="2:18">
@@ -7153,7 +7153,7 @@
         <v>5</v>
       </c>
       <c r="O65" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="P65">
         <v>60</v>
@@ -7162,7 +7162,7 @@
         <v>237</v>
       </c>
       <c r="R65" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="66" spans="2:18">
@@ -7190,7 +7190,7 @@
         <v>5</v>
       </c>
       <c r="O66" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="P66">
         <v>61</v>
@@ -7199,7 +7199,7 @@
         <v>232</v>
       </c>
       <c r="R66" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="67" spans="2:18">
@@ -7227,7 +7227,7 @@
         <v>5</v>
       </c>
       <c r="O67" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="P67">
         <v>62</v>
@@ -7236,7 +7236,7 @@
         <v>232</v>
       </c>
       <c r="R67" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="68" spans="2:18">
@@ -7264,7 +7264,7 @@
         <v>5</v>
       </c>
       <c r="O68" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="P68">
         <v>63</v>
@@ -7273,7 +7273,7 @@
         <v>232</v>
       </c>
       <c r="R68" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="69" spans="2:18">
@@ -7301,7 +7301,7 @@
         <v>5</v>
       </c>
       <c r="O69" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="P69">
         <v>64</v>
@@ -7310,7 +7310,7 @@
         <v>232</v>
       </c>
       <c r="R69" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="70" spans="2:18">
@@ -7338,7 +7338,7 @@
         <v>5</v>
       </c>
       <c r="O70" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="P70">
         <v>65</v>
@@ -7347,7 +7347,7 @@
         <v>232</v>
       </c>
       <c r="R70" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="71" spans="2:18">
@@ -7375,7 +7375,7 @@
         <v>5</v>
       </c>
       <c r="O71" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="P71">
         <v>66</v>
@@ -7384,7 +7384,7 @@
         <v>233</v>
       </c>
       <c r="R71" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="72" spans="2:18">
@@ -7412,7 +7412,7 @@
         <v>5</v>
       </c>
       <c r="O72" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="P72">
         <v>67</v>
@@ -7421,7 +7421,7 @@
         <v>233</v>
       </c>
       <c r="R72" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="73" spans="2:18">
@@ -7449,7 +7449,7 @@
         <v>5</v>
       </c>
       <c r="O73" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="P73">
         <v>68</v>
@@ -7458,7 +7458,7 @@
         <v>233</v>
       </c>
       <c r="R73" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="74" spans="2:18">
@@ -7486,7 +7486,7 @@
         <v>5</v>
       </c>
       <c r="O74" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="P74">
         <v>69</v>
@@ -7495,7 +7495,7 @@
         <v>233</v>
       </c>
       <c r="R74" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="75" spans="2:18">
@@ -7523,7 +7523,7 @@
         <v>5</v>
       </c>
       <c r="O75" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="P75">
         <v>70</v>
@@ -7532,7 +7532,7 @@
         <v>233</v>
       </c>
       <c r="R75" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -7685,7 +7685,7 @@
         <v>157</v>
       </c>
       <c r="I5" t="s">
-        <v>261</v>
+        <v>387</v>
       </c>
       <c r="K5" t="s">
         <v>80</v>
@@ -7769,7 +7769,7 @@
         <v>117</v>
       </c>
       <c r="K9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="N9" t="s">
         <v>82</v>
@@ -7851,13 +7851,13 @@
     </row>
     <row r="14" spans="1:21">
       <c r="A14" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="K14" t="s">
+        <v>291</v>
+      </c>
+      <c r="N14" t="s">
         <v>292</v>
-      </c>
-      <c r="N14" t="s">
-        <v>293</v>
       </c>
       <c r="Q14" t="s">
         <v>50</v>
@@ -7865,13 +7865,13 @@
     </row>
     <row r="15" spans="1:21">
       <c r="A15" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="K15" t="s">
         <v>291</v>
       </c>
-      <c r="K15" t="s">
-        <v>292</v>
-      </c>
       <c r="N15" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="Q15" t="s">
         <v>50</v>
@@ -7976,7 +7976,7 @@
   <sheetData>
     <row r="3" spans="1:19" ht="17.25" thickBot="1">
       <c r="A3" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="15" thickTop="1" thickBot="1">
@@ -8084,7 +8084,7 @@
     </row>
     <row r="10" spans="1:19" ht="17.25" thickBot="1">
       <c r="A10" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="15" thickTop="1" thickBot="1">
@@ -8151,7 +8151,7 @@
         <v>120</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -8170,7 +8170,7 @@
         <v>160</v>
       </c>
       <c r="M13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="S13">
         <v>-1</v>
@@ -8192,7 +8192,7 @@
         <v>160</v>
       </c>
       <c r="M14" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="S14">
         <v>-1</v>
@@ -8203,7 +8203,7 @@
         <v>120</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -8222,7 +8222,7 @@
         <v>160</v>
       </c>
       <c r="M16" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="S16">
         <v>-1</v>
@@ -8244,7 +8244,7 @@
         <v>160</v>
       </c>
       <c r="M17" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="S17">
         <v>-1</v>
@@ -8255,7 +8255,7 @@
         <v>120</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -8273,7 +8273,7 @@
         <v>160</v>
       </c>
       <c r="M19" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="S19">
         <v>-1</v>
@@ -8294,7 +8294,7 @@
         <v>160</v>
       </c>
       <c r="M20" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="S20">
         <v>-1</v>
@@ -8314,7 +8314,7 @@
         <v>160</v>
       </c>
       <c r="M23" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="S23">
         <v>-1</v>
@@ -8438,7 +8438,7 @@
         <v>94</v>
       </c>
       <c r="B12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -8446,7 +8446,7 @@
         <v>95</v>
       </c>
       <c r="B13" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -8979,7 +8979,7 @@
         <v>202</v>
       </c>
       <c r="B24" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -8987,7 +8987,7 @@
         <v>203</v>
       </c>
       <c r="B25" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -9004,7 +9004,7 @@
         <v>187</v>
       </c>
       <c r="B27" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -9141,7 +9141,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
@@ -9150,7 +9150,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
@@ -9177,7 +9177,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -9186,7 +9186,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -9195,18 +9195,18 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B13" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-22 22:43
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_DEU/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3BCA134-6F6E-46C7-B2D4-F78ECE5CD6C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EB1C8A7-4808-4116-B649-64C70DAF59A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="418">
   <si>
     <t>Unit</t>
   </si>
@@ -1246,6 +1246,96 @@
   </si>
   <si>
     <t>ELC,ELC_???[_]???*,e[_]*</t>
+  </si>
+  <si>
+    <t>IRE</t>
+  </si>
+  <si>
+    <t>g[_]*</t>
+  </si>
+  <si>
+    <t>Grid Capacity</t>
+  </si>
+  <si>
+    <t>Grid New Capacity</t>
+  </si>
+  <si>
+    <t>Sector</t>
+  </si>
+  <si>
+    <t>e_dem*</t>
+  </si>
+  <si>
+    <t>Industry and Buildings</t>
+  </si>
+  <si>
+    <t>ev_bat*</t>
+  </si>
+  <si>
+    <t>H2Prd*</t>
+  </si>
+  <si>
+    <t>e_dem*,ev_bat*,H2Prd*</t>
+  </si>
+  <si>
+    <t>e*</t>
+  </si>
+  <si>
+    <t>~tradeflow_exp</t>
+  </si>
+  <si>
+    <t>Internal variable to create Grid-level trade flows</t>
+  </si>
+  <si>
+    <t>p,c</t>
+  </si>
+  <si>
+    <t>~tradeflow_imp</t>
+  </si>
+  <si>
+    <t>ELC_???[_]???*,e[_]*</t>
+  </si>
+  <si>
+    <t>VerveStacks</t>
+  </si>
+  <si>
+    <t>Tech_origin</t>
+  </si>
+  <si>
+    <t>ep_*</t>
+  </si>
+  <si>
+    <t>GEM_operating</t>
+  </si>
+  <si>
+    <t>en_pc_*</t>
+  </si>
+  <si>
+    <t>GEM_pre-constr</t>
+  </si>
+  <si>
+    <t>ep_m_*</t>
+  </si>
+  <si>
+    <t>GEM_mothballed</t>
+  </si>
+  <si>
+    <t>en_a_*</t>
+  </si>
+  <si>
+    <t>GEM_announced</t>
+  </si>
+  <si>
+    <t>en_can_*</t>
+  </si>
+  <si>
+    <t>GEM_cancelled</t>
+  </si>
+  <si>
+    <t>en_she_*</t>
+  </si>
+  <si>
+    <t>GEM_shelved</t>
   </si>
 </sst>
 </file>
@@ -3821,7 +3911,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10ADB714-E6AA-4E3E-B77B-62B65BA0E218}">
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.86328125" bestFit="1" customWidth="1"/>
@@ -4509,6 +4599,116 @@
       </c>
       <c r="C56" t="s">
         <v>114</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" t="s">
+        <v>392</v>
+      </c>
+      <c r="B57" t="s">
+        <v>393</v>
+      </c>
+      <c r="C57" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
+        <v>392</v>
+      </c>
+      <c r="B58" t="s">
+        <v>395</v>
+      </c>
+      <c r="C58" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" t="s">
+        <v>392</v>
+      </c>
+      <c r="B59" t="s">
+        <v>396</v>
+      </c>
+      <c r="C59" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" t="s">
+        <v>405</v>
+      </c>
+      <c r="B60" t="s">
+        <v>120</v>
+      </c>
+      <c r="C60" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
+        <v>405</v>
+      </c>
+      <c r="B61" t="s">
+        <v>406</v>
+      </c>
+      <c r="C61" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" t="s">
+        <v>405</v>
+      </c>
+      <c r="B62" t="s">
+        <v>408</v>
+      </c>
+      <c r="C62" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63" t="s">
+        <v>405</v>
+      </c>
+      <c r="B63" t="s">
+        <v>410</v>
+      </c>
+      <c r="C63" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" t="s">
+        <v>405</v>
+      </c>
+      <c r="B64" t="s">
+        <v>412</v>
+      </c>
+      <c r="C64" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>405</v>
+      </c>
+      <c r="B65" t="s">
+        <v>414</v>
+      </c>
+      <c r="C65" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>405</v>
+      </c>
+      <c r="B66" t="s">
+        <v>416</v>
+      </c>
+      <c r="C66" t="s">
+        <v>417</v>
       </c>
     </row>
   </sheetData>
@@ -7548,7 +7748,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet19"/>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="13.86328125" bestFit="1" customWidth="1"/>
@@ -7877,6 +8077,97 @@
         <v>50</v>
       </c>
     </row>
+    <row r="16" spans="1:21">
+      <c r="A16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>388</v>
+      </c>
+      <c r="D16" t="s">
+        <v>389</v>
+      </c>
+      <c r="K16" t="s">
+        <v>8</v>
+      </c>
+      <c r="N16" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
+      <c r="A17" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" t="s">
+        <v>388</v>
+      </c>
+      <c r="D17" t="s">
+        <v>389</v>
+      </c>
+      <c r="K17" t="s">
+        <v>8</v>
+      </c>
+      <c r="N17" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17">
+      <c r="A18" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D18" t="s">
+        <v>397</v>
+      </c>
+      <c r="I18" t="s">
+        <v>398</v>
+      </c>
+      <c r="K18" t="s">
+        <v>80</v>
+      </c>
+      <c r="N18" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17">
+      <c r="A19" t="s">
+        <v>161</v>
+      </c>
+      <c r="I19" t="s">
+        <v>403</v>
+      </c>
+      <c r="K19" t="s">
+        <v>80</v>
+      </c>
+      <c r="N19" t="s">
+        <v>399</v>
+      </c>
+      <c r="P19" t="s">
+        <v>400</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="I20" t="s">
+        <v>403</v>
+      </c>
+      <c r="K20" t="s">
+        <v>80</v>
+      </c>
+      <c r="N20" t="s">
+        <v>402</v>
+      </c>
+      <c r="P20" t="s">
+        <v>400</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>401</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="T4:U4"/>

</xml_diff>